<commit_message>
Actualización automática 2026-01-08 17:30:09
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R24"/>
+  <dimension ref="A1:R25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1818,137 +1818,197 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
           <t>VIEJO RIVAS MAYRA ANABELLE</t>
         </is>
       </c>
-      <c r="C23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R23" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>0 de 22</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>0 de 22</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>0 de 22</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>0 de 22</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>0 de 22</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>0 de 22</t>
-        </is>
-      </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>0 de 22</t>
-        </is>
-      </c>
-      <c r="J24" s="3" t="inlineStr">
-        <is>
-          <t>0 de 22</t>
-        </is>
-      </c>
-      <c r="K24" s="3" t="inlineStr">
-        <is>
-          <t>0 de 22</t>
-        </is>
-      </c>
-      <c r="L24" s="3" t="inlineStr">
-        <is>
-          <t>0 de 22</t>
-        </is>
-      </c>
-      <c r="M24" s="3" t="inlineStr">
-        <is>
-          <t>0 de 22</t>
-        </is>
-      </c>
-      <c r="N24" s="3" t="inlineStr">
-        <is>
-          <t>0 de 22</t>
-        </is>
-      </c>
-      <c r="O24" s="3" t="inlineStr">
-        <is>
-          <t>0 de 22</t>
-        </is>
-      </c>
-      <c r="P24" s="3" t="inlineStr">
-        <is>
-          <t>0 de 22</t>
-        </is>
-      </c>
-      <c r="Q24" s="3" t="inlineStr">
-        <is>
-          <t>0 de 22</t>
-        </is>
-      </c>
-      <c r="R24" s="3" t="inlineStr">
-        <is>
-          <t>0 de 22</t>
+      <c r="C24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0 de 23</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>0 de 23</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>0 de 23</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>0 de 23</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>0 de 23</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>0 de 23</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>0 de 23</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>0 de 23</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>0 de 23</t>
+        </is>
+      </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>0 de 23</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>0 de 23</t>
+        </is>
+      </c>
+      <c r="N25" s="3" t="inlineStr">
+        <is>
+          <t>0 de 23</t>
+        </is>
+      </c>
+      <c r="O25" s="3" t="inlineStr">
+        <is>
+          <t>0 de 23</t>
+        </is>
+      </c>
+      <c r="P25" s="3" t="inlineStr">
+        <is>
+          <t>0 de 23</t>
+        </is>
+      </c>
+      <c r="Q25" s="3" t="inlineStr">
+        <is>
+          <t>0 de 23</t>
+        </is>
+      </c>
+      <c r="R25" s="3" t="inlineStr">
+        <is>
+          <t>0 de 23</t>
         </is>
       </c>
     </row>
@@ -1963,7 +2023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2371,11 +2431,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>3896.18</v>
+        <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>0</v>
@@ -2398,11 +2458,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0</v>
+        <v>3896.18</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>0</v>
@@ -2425,7 +2485,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -2435,7 +2495,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>838.7</v>
+        <v>0</v>
       </c>
       <c r="F17" s="2" t="n">
         <v>0</v>
@@ -2452,17 +2512,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>326.73</v>
+        <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0</v>
+        <v>838.7</v>
       </c>
       <c r="F18" s="2" t="n">
         <v>0</v>
@@ -2479,17 +2539,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1015.74</v>
+        <v>326.73</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>1218.02</v>
+        <v>0</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>-591.61</v>
+        <v>0</v>
       </c>
       <c r="F19" s="2" t="n">
         <v>0</v>
@@ -2506,17 +2566,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0</v>
+        <v>1015.74</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0</v>
+        <v>1218.02</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>2963.59</v>
+        <v>-591.61</v>
       </c>
       <c r="F20" s="2" t="n">
         <v>0</v>
@@ -2533,7 +2593,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -2543,7 +2603,7 @@
         <v>0</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>232.74</v>
+        <v>2963.59</v>
       </c>
       <c r="F21" s="2" t="n">
         <v>0</v>
@@ -2560,23 +2620,23 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1115.07</v>
+        <v>0</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>388.8</v>
+        <v>232.74</v>
       </c>
       <c r="F22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -2587,39 +2647,66 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>1115.07</v>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>388.8</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
           <t>VIEJO RIVAS MAYRA ANABELLE</t>
         </is>
       </c>
-      <c r="C23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="C24" s="4" t="n">
+      <c r="C24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="C25" s="4" t="n">
         <v>18337.91</v>
       </c>
-      <c r="D24" s="4" t="n">
+      <c r="D25" s="4" t="n">
         <v>3750.24</v>
       </c>
-      <c r="E24" s="4" t="n">
+      <c r="E25" s="4" t="n">
         <v>16490.86</v>
       </c>
-      <c r="F24" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="4" t="n">
+      <c r="F25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="4" t="n">
         <v>1000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-01-09 12:30:07
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R26"/>
+  <dimension ref="A1:R35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -558,7 +558,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ARMIJOS SALINAS LUIS CLAUDIO</t>
+          <t>ALTAMIRANO VILLAVICENCIO JUAN ALEJANDRO</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -618,7 +618,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ASES GAVILANEZ FAUSTO HERNAN</t>
+          <t>ARMIJOS SALINAS LUIS CLAUDIO</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -678,7 +678,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BARROS YUNGA DIEGO VINICIO</t>
+          <t>ASES GAVILANEZ FAUSTO HERNAN</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -738,7 +738,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BRAVO MONTENEGRO DANIEL ANDRES</t>
+          <t>BARROS YUNGA DIEGO VINICIO</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -798,7 +798,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BRITO CARDENAS RUTH CECILIA</t>
+          <t>BRAVO MONTENEGRO DANIEL ANDRES</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>COELLO TRONCOSO JOSE GREGORIO</t>
+          <t>BRITO CARDENAS RUTH CECILIA</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -918,7 +918,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
+          <t>COELLO TRONCOSO JOSE GREGORIO</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -978,7 +978,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
+          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
+          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
+          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
+          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
+          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1732,13 +1732,13 @@
         <v>0</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>50.24</v>
+        <v>0</v>
       </c>
       <c r="N21" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O21" s="2" t="n">
-        <v>3704.28</v>
+        <v>0</v>
       </c>
       <c r="P21" s="2" t="n">
         <v>0</v>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>PACHAR TAPIA ELIANA DE LOS ANGELES</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1878,7 +1878,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1938,137 +1938,677 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="2" t="n">
+        <v>50.24</v>
+      </c>
+      <c r="N28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="2" t="n">
+        <v>3704.28</v>
+      </c>
+      <c r="P28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R29" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R30" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
           <t>VIEJO RIVAS MAYRA ANABELLE</t>
         </is>
       </c>
-      <c r="C25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R25" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>0 de 24</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>0 de 24</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>0 de 24</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>0 de 24</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>0 de 24</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>0 de 24</t>
-        </is>
-      </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>0 de 24</t>
-        </is>
-      </c>
-      <c r="J26" s="3" t="inlineStr">
-        <is>
-          <t>0 de 24</t>
-        </is>
-      </c>
-      <c r="K26" s="3" t="inlineStr">
-        <is>
-          <t>0 de 24</t>
-        </is>
-      </c>
-      <c r="L26" s="3" t="inlineStr">
-        <is>
-          <t>0 de 24</t>
-        </is>
-      </c>
-      <c r="M26" s="3" t="inlineStr">
-        <is>
-          <t>1 de 24</t>
-        </is>
-      </c>
-      <c r="N26" s="3" t="inlineStr">
-        <is>
-          <t>0 de 24</t>
-        </is>
-      </c>
-      <c r="O26" s="3" t="inlineStr">
-        <is>
-          <t>1 de 24</t>
-        </is>
-      </c>
-      <c r="P26" s="3" t="inlineStr">
-        <is>
-          <t>0 de 24</t>
-        </is>
-      </c>
-      <c r="Q26" s="3" t="inlineStr">
-        <is>
-          <t>0 de 24</t>
-        </is>
-      </c>
-      <c r="R26" s="3" t="inlineStr">
-        <is>
-          <t>0 de 24</t>
+      <c r="C33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>VIVANCO MALDONADO SILVANA MARILY</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0 de 33</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>0 de 33</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>0 de 33</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>0 de 33</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>0 de 33</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>0 de 33</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>0 de 33</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>0 de 33</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>0 de 33</t>
+        </is>
+      </c>
+      <c r="L35" s="3" t="inlineStr">
+        <is>
+          <t>0 de 33</t>
+        </is>
+      </c>
+      <c r="M35" s="3" t="inlineStr">
+        <is>
+          <t>1 de 33</t>
+        </is>
+      </c>
+      <c r="N35" s="3" t="inlineStr">
+        <is>
+          <t>0 de 33</t>
+        </is>
+      </c>
+      <c r="O35" s="3" t="inlineStr">
+        <is>
+          <t>1 de 33</t>
+        </is>
+      </c>
+      <c r="P35" s="3" t="inlineStr">
+        <is>
+          <t>0 de 33</t>
+        </is>
+      </c>
+      <c r="Q35" s="3" t="inlineStr">
+        <is>
+          <t>0 de 33</t>
+        </is>
+      </c>
+      <c r="R35" s="3" t="inlineStr">
+        <is>
+          <t>0 de 33</t>
         </is>
       </c>
     </row>
@@ -2083,7 +2623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2140,17 +2680,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ARMIJOS SALINAS LUIS CLAUDIO</t>
+          <t>ALTAMIRANO VILLAVICENCIO JUAN ALEJANDRO</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0</v>
+        <v>848.76</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>797.36</v>
+        <v>785.09</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1347.49</v>
+        <v>0</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>0</v>
@@ -2167,17 +2707,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ASES GAVILANEZ FAUSTO HERNAN</t>
+          <t>ARMIJOS SALINAS LUIS CLAUDIO</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0</v>
+        <v>797.36</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0</v>
+        <v>1347.49</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>0</v>
@@ -2194,11 +2734,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BARROS YUNGA DIEGO VINICIO</t>
+          <t>ASES GAVILANEZ FAUSTO HERNAN</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>17.99</v>
+        <v>0</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>0</v>
@@ -2221,11 +2761,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BRAVO MONTENEGRO DANIEL ANDRES</t>
+          <t>BARROS YUNGA DIEGO VINICIO</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0</v>
+        <v>17.99</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>0</v>
@@ -2248,7 +2788,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BRITO CARDENAS RUTH CECILIA</t>
+          <t>BRAVO MONTENEGRO DANIEL ANDRES</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -2275,7 +2815,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>COELLO TRONCOSO JOSE GREGORIO</t>
+          <t>BRITO CARDENAS RUTH CECILIA</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -2302,7 +2842,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
+          <t>COELLO TRONCOSO JOSE GREGORIO</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -2329,14 +2869,14 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
+          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3992.9</v>
+        <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>1631.15</v>
+        <v>0</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0</v>
@@ -2356,7 +2896,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
+          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -2383,14 +2923,14 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
+          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>252.25</v>
+        <v>3992.9</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0</v>
+        <v>1631.15</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>0</v>
@@ -2410,23 +2950,23 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
+          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>7662.57</v>
+        <v>0</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>4874.94</v>
+        <v>0</v>
       </c>
       <c r="F12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="13">
@@ -2437,7 +2977,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
+          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -2447,7 +2987,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>6342.22</v>
+        <v>0</v>
       </c>
       <c r="F13" s="2" t="n">
         <v>0</v>
@@ -2464,17 +3004,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>58.48</v>
+        <v>252.25</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>103.71</v>
+        <v>0</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>93.98999999999999</v>
+        <v>0</v>
       </c>
       <c r="F14" s="2" t="n">
         <v>0</v>
@@ -2491,17 +3031,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0</v>
+        <v>7662.57</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0</v>
+        <v>4874.94</v>
       </c>
       <c r="F15" s="2" t="n">
         <v>0</v>
@@ -2518,17 +3058,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>3896.18</v>
+        <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0</v>
+        <v>6342.22</v>
       </c>
       <c r="F16" s="2" t="n">
         <v>0</v>
@@ -2545,17 +3085,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0</v>
+        <v>58.48</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0</v>
+        <v>103.71</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0</v>
+        <v>93.98999999999999</v>
       </c>
       <c r="F17" s="2" t="n">
         <v>0</v>
@@ -2572,7 +3112,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -2582,7 +3122,7 @@
         <v>0</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>838.7</v>
+        <v>0</v>
       </c>
       <c r="F18" s="2" t="n">
         <v>0</v>
@@ -2599,11 +3139,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>326.73</v>
+        <v>3896.18</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>0</v>
@@ -2626,17 +3166,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1015.74</v>
+        <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>1218.02</v>
+        <v>0</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>-591.61</v>
+        <v>0</v>
       </c>
       <c r="F20" s="2" t="n">
         <v>0</v>
@@ -2653,23 +3193,23 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>3130.46</v>
+        <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>765.08</v>
+        <v>0</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>8877.290000000001</v>
+        <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>3754.52</v>
+        <v>0</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -2680,7 +3220,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -2690,7 +3230,7 @@
         <v>0</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>2963.59</v>
+        <v>838.7</v>
       </c>
       <c r="F22" s="2" t="n">
         <v>0</v>
@@ -2707,7 +3247,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>PACHAR TAPIA ELIANA DE LOS ANGELES</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -2717,7 +3257,7 @@
         <v>0</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>232.74</v>
+        <v>0</v>
       </c>
       <c r="F23" s="2" t="n">
         <v>0</v>
@@ -2734,23 +3274,23 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1115.07</v>
+        <v>326.73</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>388.8</v>
+        <v>0</v>
       </c>
       <c r="F24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -2761,40 +3301,283 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>3628.38</v>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>2179.48</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>1015.74</v>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>1218.02</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>-591.61</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>3130.46</v>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>765.08</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>8877.290000000001</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>3754.52</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>2963.59</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>232.74</v>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>1115.07</v>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>388.8</v>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
           <t>VIEJO RIVAS MAYRA ANABELLE</t>
         </is>
       </c>
-      <c r="C25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="C26" s="4" t="n">
-        <v>21468.37</v>
-      </c>
-      <c r="D26" s="4" t="n">
-        <v>4515.32</v>
-      </c>
-      <c r="E26" s="4" t="n">
-        <v>25368.15</v>
-      </c>
-      <c r="F26" s="4" t="n">
+      <c r="C33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>VIVANCO MALDONADO SILVANA MARILY</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>1443.42</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>1062.8</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>673.6900000000001</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="C35" s="4" t="n">
+        <v>27388.93</v>
+      </c>
+      <c r="D35" s="4" t="n">
+        <v>8542.690000000001</v>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>26041.84</v>
+      </c>
+      <c r="F35" s="4" t="n">
         <v>3754.52</v>
       </c>
-      <c r="G26" s="4" t="n">
-        <v>3000</v>
+      <c r="G35" s="4" t="n">
+        <v>5000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-01-09 13:30:07
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R35"/>
+  <dimension ref="A1:R48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -558,7 +558,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ALTAMIRANO VILLAVICENCIO JUAN ALEJANDRO</t>
+          <t>ALTAMIRANO ARIAS LUCIA ELIZABETH</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -618,7 +618,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ARMIJOS SALINAS LUIS CLAUDIO</t>
+          <t>ALTAMIRANO VILLAVICENCIO JUAN ALEJANDRO</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -678,7 +678,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ASES GAVILANEZ FAUSTO HERNAN</t>
+          <t>ALVAREZ SAAVEDRA EDWIN GEOVANNY</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -738,7 +738,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BARROS YUNGA DIEGO VINICIO</t>
+          <t>ARMIJOS SALINAS LUIS CLAUDIO</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -798,7 +798,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BRAVO MONTENEGRO DANIEL ANDRES</t>
+          <t>ASES GAVILANEZ FAUSTO HERNAN</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BRITO CARDENAS RUTH CECILIA</t>
+          <t>BARROS YUNGA DIEGO VINICIO</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -918,7 +918,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>COELLO TRONCOSO JOSE GREGORIO</t>
+          <t>BRAVO MONTENEGRO DANIEL ANDRES</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -978,7 +978,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
+          <t>BRITO CARDENAS RUTH CECILIA</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
+          <t>COELLO TRONCOSO JOSE GREGORIO</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
+          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
+          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
+          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
+          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
+          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
+          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1732,7 +1732,7 @@
         <v>0</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>0</v>
+        <v>1694.28</v>
       </c>
       <c r="N21" s="2" t="n">
         <v>0</v>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>JUAREZ FLORES JORGE WILLIAMS</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PACHAR TAPIA ELIANA DE LOS ANGELES</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1878,7 +1878,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>MENA COSTA GUIDO LENNIN</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -1998,7 +1998,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>MORALES GRACIELA ENITH</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2152,13 +2152,13 @@
         <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>50.24</v>
+        <v>0</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O28" s="2" t="n">
-        <v>3704.28</v>
+        <v>0</v>
       </c>
       <c r="P28" s="2" t="n">
         <v>0</v>
@@ -2178,7 +2178,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2238,7 +2238,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>PACHAR TAPIA ELIANA DE LOS ANGELES</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>VIEJO RIVAS MAYRA ANABELLE</t>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2478,137 +2478,917 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R35" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" s="2" t="n">
+        <v>50.24</v>
+      </c>
+      <c r="N36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" s="2" t="n">
+        <v>3704.28</v>
+      </c>
+      <c r="P36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R38" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R39" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R40" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R41" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>SOPLIN MENDOZA TABITA</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R42" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R43" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" s="2" t="n">
+        <v>24.88</v>
+      </c>
+      <c r="P44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R44" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R45" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>VIEJO RIVAS MAYRA ANABELLE</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R46" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R34" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>0 de 33</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>0 de 33</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>0 de 33</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>0 de 33</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t>0 de 33</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>0 de 33</t>
-        </is>
-      </c>
-      <c r="I35" s="3" t="inlineStr">
-        <is>
-          <t>0 de 33</t>
-        </is>
-      </c>
-      <c r="J35" s="3" t="inlineStr">
-        <is>
-          <t>0 de 33</t>
-        </is>
-      </c>
-      <c r="K35" s="3" t="inlineStr">
-        <is>
-          <t>0 de 33</t>
-        </is>
-      </c>
-      <c r="L35" s="3" t="inlineStr">
-        <is>
-          <t>0 de 33</t>
-        </is>
-      </c>
-      <c r="M35" s="3" t="inlineStr">
-        <is>
-          <t>1 de 33</t>
-        </is>
-      </c>
-      <c r="N35" s="3" t="inlineStr">
-        <is>
-          <t>0 de 33</t>
-        </is>
-      </c>
-      <c r="O35" s="3" t="inlineStr">
-        <is>
-          <t>1 de 33</t>
-        </is>
-      </c>
-      <c r="P35" s="3" t="inlineStr">
-        <is>
-          <t>0 de 33</t>
-        </is>
-      </c>
-      <c r="Q35" s="3" t="inlineStr">
-        <is>
-          <t>0 de 33</t>
-        </is>
-      </c>
-      <c r="R35" s="3" t="inlineStr">
-        <is>
-          <t>0 de 33</t>
+      <c r="C47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R47" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0 de 46</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>0 de 46</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>0 de 46</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>0 de 46</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>0 de 46</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>0 de 46</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>0 de 46</t>
+        </is>
+      </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>0 de 46</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr">
+        <is>
+          <t>0 de 46</t>
+        </is>
+      </c>
+      <c r="L48" s="3" t="inlineStr">
+        <is>
+          <t>0 de 46</t>
+        </is>
+      </c>
+      <c r="M48" s="3" t="inlineStr">
+        <is>
+          <t>2 de 46</t>
+        </is>
+      </c>
+      <c r="N48" s="3" t="inlineStr">
+        <is>
+          <t>0 de 46</t>
+        </is>
+      </c>
+      <c r="O48" s="3" t="inlineStr">
+        <is>
+          <t>2 de 46</t>
+        </is>
+      </c>
+      <c r="P48" s="3" t="inlineStr">
+        <is>
+          <t>0 de 46</t>
+        </is>
+      </c>
+      <c r="Q48" s="3" t="inlineStr">
+        <is>
+          <t>0 de 46</t>
+        </is>
+      </c>
+      <c r="R48" s="3" t="inlineStr">
+        <is>
+          <t>0 de 46</t>
         </is>
       </c>
     </row>
@@ -2623,7 +3403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2680,23 +3460,23 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ALTAMIRANO VILLAVICENCIO JUAN ALEJANDRO</t>
+          <t>ALTAMIRANO ARIAS LUCIA ELIZABETH</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>848.76</v>
+        <v>6405.28</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>785.09</v>
+        <v>0</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0</v>
+        <v>6526.56</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="3">
@@ -2707,17 +3487,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ARMIJOS SALINAS LUIS CLAUDIO</t>
+          <t>ALTAMIRANO VILLAVICENCIO JUAN ALEJANDRO</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0</v>
+        <v>848.76</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>797.36</v>
+        <v>785.09</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1347.49</v>
+        <v>0</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>0</v>
@@ -2734,7 +3514,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ASES GAVILANEZ FAUSTO HERNAN</t>
+          <t>ALVAREZ SAAVEDRA EDWIN GEOVANNY</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -2744,7 +3524,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0</v>
+        <v>661.5</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>0</v>
@@ -2761,17 +3541,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BARROS YUNGA DIEGO VINICIO</t>
+          <t>ARMIJOS SALINAS LUIS CLAUDIO</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>17.99</v>
+        <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0</v>
+        <v>797.36</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0</v>
+        <v>1347.49</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>0</v>
@@ -2788,7 +3568,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BRAVO MONTENEGRO DANIEL ANDRES</t>
+          <t>ASES GAVILANEZ FAUSTO HERNAN</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -2815,11 +3595,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BRITO CARDENAS RUTH CECILIA</t>
+          <t>BARROS YUNGA DIEGO VINICIO</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0</v>
+        <v>17.99</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>0</v>
@@ -2842,7 +3622,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>COELLO TRONCOSO JOSE GREGORIO</t>
+          <t>BRAVO MONTENEGRO DANIEL ANDRES</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -2869,7 +3649,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
+          <t>BRITO CARDENAS RUTH CECILIA</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -2896,7 +3676,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
+          <t>COELLO TRONCOSO JOSE GREGORIO</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -2923,14 +3703,14 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
+          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>3992.9</v>
+        <v>0</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1631.15</v>
+        <v>0</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>0</v>
@@ -2950,7 +3730,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
+          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -2966,7 +3746,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -2977,14 +3757,14 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
+          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0</v>
+        <v>3992.9</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0</v>
+        <v>1631.15</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>0</v>
@@ -3004,11 +3784,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
+          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>252.25</v>
+        <v>0</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>0</v>
@@ -3020,7 +3800,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="15">
@@ -3031,17 +3811,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
+          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>7662.57</v>
+        <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>4874.94</v>
+        <v>0</v>
       </c>
       <c r="F15" s="2" t="n">
         <v>0</v>
@@ -3058,17 +3838,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
+          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0</v>
+        <v>252.25</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>6342.22</v>
+        <v>0</v>
       </c>
       <c r="F16" s="2" t="n">
         <v>0</v>
@@ -3085,17 +3865,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>58.48</v>
+        <v>7662.57</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>103.71</v>
+        <v>0</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>93.98999999999999</v>
+        <v>4874.94</v>
       </c>
       <c r="F17" s="2" t="n">
         <v>0</v>
@@ -3112,23 +3892,23 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0</v>
+        <v>1891.36</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0</v>
+        <v>1058.37</v>
       </c>
       <c r="F18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="19">
@@ -3139,17 +3919,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>3896.18</v>
+        <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>0</v>
+        <v>6342.22</v>
       </c>
       <c r="F19" s="2" t="n">
         <v>0</v>
@@ -3166,17 +3946,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0</v>
+        <v>58.48</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0</v>
+        <v>103.71</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0</v>
+        <v>93.98999999999999</v>
       </c>
       <c r="F20" s="2" t="n">
         <v>0</v>
@@ -3193,11 +3973,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0</v>
+        <v>89.56</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>0</v>
@@ -3206,7 +3986,7 @@
         <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0</v>
+        <v>1694.28</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>0</v>
@@ -3220,17 +4000,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>JUAREZ FLORES JORGE WILLIAMS</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0</v>
+        <v>3066.76</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0</v>
+        <v>1770.09</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>838.7</v>
+        <v>381.6</v>
       </c>
       <c r="F22" s="2" t="n">
         <v>0</v>
@@ -3247,7 +4027,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PACHAR TAPIA ELIANA DE LOS ANGELES</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -3274,11 +4054,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>MENA COSTA GUIDO LENNIN</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>326.73</v>
+        <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>0</v>
@@ -3301,11 +4081,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0</v>
+        <v>3896.18</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>0</v>
@@ -3328,14 +4108,14 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>3628.38</v>
+        <v>0</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>2179.48</v>
+        <v>0</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>0</v>
@@ -3344,7 +4124,7 @@
         <v>0</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -3355,17 +4135,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>MORALES GRACIELA ENITH</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>1015.74</v>
+        <v>829.4400000000001</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>1218.02</v>
+        <v>0</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>-591.61</v>
+        <v>0</v>
       </c>
       <c r="F27" s="2" t="n">
         <v>0</v>
@@ -3382,23 +4162,23 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>3130.46</v>
+        <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>765.08</v>
+        <v>0</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>8877.290000000001</v>
+        <v>0</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>3754.52</v>
+        <v>0</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -3409,7 +4189,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -3419,7 +4199,7 @@
         <v>0</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0</v>
+        <v>838.7</v>
       </c>
       <c r="F29" s="2" t="n">
         <v>0</v>
@@ -3436,7 +4216,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -3446,7 +4226,7 @@
         <v>0</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>2963.59</v>
+        <v>0</v>
       </c>
       <c r="F30" s="2" t="n">
         <v>0</v>
@@ -3463,7 +4243,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>PACHAR TAPIA ELIANA DE LOS ANGELES</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -3473,7 +4253,7 @@
         <v>0</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>232.74</v>
+        <v>0</v>
       </c>
       <c r="F31" s="2" t="n">
         <v>0</v>
@@ -3490,23 +4270,23 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>1115.07</v>
+        <v>326.73</v>
       </c>
       <c r="D32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>388.8</v>
+        <v>0</v>
       </c>
       <c r="F32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -3517,7 +4297,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>VIEJO RIVAS MAYRA ANABELLE</t>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -3544,40 +4324,391 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>3628.38</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>2179.48</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>1015.74</v>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>1218.02</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>-591.61</v>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>3130.46</v>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>765.08</v>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>8877.290000000001</v>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>3754.52</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>165.48</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>255.57</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>2963.59</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>6889.32</v>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>SOPLIN MENDOZA TABITA</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>232.74</v>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>269.28</v>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>24.88</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="n">
+        <v>1115.07</v>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>388.8</v>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>VIEJO RIVAS MAYRA ANABELLE</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C34" s="2" t="n">
+      <c r="C47" s="2" t="n">
         <v>1443.42</v>
       </c>
-      <c r="D34" s="2" t="n">
+      <c r="D47" s="2" t="n">
         <v>1062.8</v>
       </c>
-      <c r="E34" s="2" t="n">
+      <c r="E47" s="2" t="n">
         <v>673.6900000000001</v>
       </c>
-      <c r="F34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G34" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="C35" s="4" t="n">
-        <v>27388.93</v>
-      </c>
-      <c r="D35" s="4" t="n">
-        <v>8542.690000000001</v>
-      </c>
-      <c r="E35" s="4" t="n">
-        <v>26041.84</v>
-      </c>
-      <c r="F35" s="4" t="n">
-        <v>3754.52</v>
-      </c>
-      <c r="G35" s="4" t="n">
-        <v>5000</v>
+      <c r="F47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="C48" s="4" t="n">
+        <v>44938.57</v>
+      </c>
+      <c r="D48" s="4" t="n">
+        <v>12369.62</v>
+      </c>
+      <c r="E48" s="4" t="n">
+        <v>34925.44</v>
+      </c>
+      <c r="F48" s="4" t="n">
+        <v>5473.68</v>
+      </c>
+      <c r="G48" s="4" t="n">
+        <v>12500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-01-28 13:30:11
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2970,7 +2970,7 @@
         <v>0</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>457.92</v>
+        <v>3291.84</v>
       </c>
       <c r="E42" s="2" t="n">
         <v>0</v>
@@ -4699,7 +4699,7 @@
         <v>0</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>457.92</v>
+        <v>3291.84</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>2500</v>
@@ -4726,7 +4726,7 @@
         <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>457.92</v>
+        <v>3291.84</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>1500</v>
@@ -4905,7 +4905,7 @@
         <v>50329.29</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>24178.8</v>
+        <v>29846.64</v>
       </c>
       <c r="G53" s="4" t="n">
         <v>24500</v>
@@ -4980,13 +4980,13 @@
         <v>2600</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>457.92</v>
+        <v>3291.84</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>2142.08</v>
+        <v>-691.8400000000001</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.1761230769230769</v>
+        <v>1.266092307692308</v>
       </c>
     </row>
     <row r="3">
@@ -5215,13 +5215,13 @@
         <v>25022</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>11270.73</v>
+        <v>14104.65</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>13751.27</v>
+        <v>10917.35</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.4504328191191751</v>
+        <v>0.5636899528414996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-01-28 15:30:11
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -1734,7 +1734,7 @@
         <v>0</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>0</v>
+        <v>616.95</v>
       </c>
       <c r="M21" s="2" t="n">
         <v>1694.28</v>
@@ -2706,7 +2706,7 @@
         <v>3704.28</v>
       </c>
       <c r="P37" s="2" t="n">
-        <v>15.25</v>
+        <v>400.69</v>
       </c>
       <c r="Q37" s="2" t="n">
         <v>0</v>
@@ -3423,7 +3423,7 @@
       </c>
       <c r="L49" s="3" t="inlineStr">
         <is>
-          <t>1 de 47</t>
+          <t>2 de 47</t>
         </is>
       </c>
       <c r="M49" s="3" t="inlineStr">
@@ -4078,7 +4078,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>1694.28</v>
+        <v>2311.23</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>1500</v>
@@ -4537,7 +4537,7 @@
         <v>8877.290000000001</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>5043.12</v>
+        <v>5428.56</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>2000</v>
@@ -4564,7 +4564,7 @@
         <v>8877.290000000001</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>5043.12</v>
+        <v>5428.56</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>3000</v>
@@ -4905,7 +4905,7 @@
         <v>50329.29</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>29846.64</v>
+        <v>31234.47</v>
       </c>
       <c r="G53" s="4" t="n">
         <v>24500</v>
@@ -5100,10 +5100,10 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>25.17</v>
+        <v>1027.56</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-25.17</v>
+        <v>-1027.56</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0</v>
@@ -5215,13 +5215,13 @@
         <v>25022</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>14104.65</v>
+        <v>15107.04</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>10917.35</v>
+        <v>9914.959999999999</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.5636899528414996</v>
+        <v>0.6037502997362322</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-03 13:30:11
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -597,7 +597,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>0</v>
+        <v>57.28</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>0</v>
@@ -3488,7 +3488,7 @@
       </c>
       <c r="M50" s="3" t="inlineStr">
         <is>
-          <t>0 de 48</t>
+          <t>1 de 48</t>
         </is>
       </c>
       <c r="N50" s="3" t="inlineStr">
@@ -3598,7 +3598,7 @@
         <v>2444.08</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0</v>
+        <v>57.28</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>2500</v>
@@ -3625,7 +3625,7 @@
         <v>2444.08</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0</v>
+        <v>57.28</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>2000</v>
@@ -4992,7 +4992,7 @@
         <v>33603.74</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>153.9</v>
+        <v>268.46</v>
       </c>
       <c r="G54" s="4" t="n">
         <v>24500</v>

</xml_diff>

<commit_message>
Actualización automática 2026-02-04 15:30:13
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R50"/>
+  <dimension ref="A1:R51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>COELLO TRONCOSO JOSE GREGORIO</t>
+          <t>BURNEO CELI LEYDI TATIANA</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
+          <t>COELLO TRONCOSO JOSE GREGORIO</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
+          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
+          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
+          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
+          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
+          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
+          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
+          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
+          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>JIMENEZ GORDILLO LADY KARINA</t>
+          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>JUAREZ FLORES JORGE WILLIAMS</t>
+          <t>JIMENEZ GORDILLO LADY KARINA</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>LEMA ESPINOZA MANUEL MARIA</t>
+          <t>JUAREZ FLORES JORGE WILLIAMS</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>LEMA ESPINOZA MANUEL MARIA</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>MENA COSTA GUIDO LENNIN</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MENA COSTA GUIDO LENNIN</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MORALES GRACIELA ENITH</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MORALES GRACIELA ENITH</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PACHAR TAPIA ELIANA DE LOS ANGELES</t>
+          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>PACHAR TAPIA ELIANA DE LOS ANGELES</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2505,7 +2505,7 @@
         <v>0</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>153.9</v>
+        <v>0</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0</v>
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2565,7 +2565,7 @@
         <v>0</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>0</v>
+        <v>153.9</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0</v>
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2757,7 +2757,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>96.37</v>
+        <v>0</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>0</v>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2817,7 +2817,7 @@
         <v>0</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>0</v>
+        <v>96.37</v>
       </c>
       <c r="N39" s="2" t="n">
         <v>0</v>
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>SOPLIN MENDOZA TABITA</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>VIEJO RIVAS MAYRA ANABELLE</t>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,137 +3383,197 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
+          <t>VIEJO RIVAS MAYRA ANABELLE</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R49" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C49" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D49" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E49" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F49" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G49" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I49" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J49" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K49" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L49" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M49" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N49" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O49" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P49" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q49" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R49" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t>0 de 48</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>0 de 48</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="inlineStr">
-        <is>
-          <t>0 de 48</t>
-        </is>
-      </c>
-      <c r="F50" s="3" t="inlineStr">
-        <is>
-          <t>0 de 48</t>
-        </is>
-      </c>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>0 de 48</t>
-        </is>
-      </c>
-      <c r="H50" s="3" t="inlineStr">
-        <is>
-          <t>0 de 48</t>
-        </is>
-      </c>
-      <c r="I50" s="3" t="inlineStr">
-        <is>
-          <t>1 de 48</t>
-        </is>
-      </c>
-      <c r="J50" s="3" t="inlineStr">
-        <is>
-          <t>0 de 48</t>
-        </is>
-      </c>
-      <c r="K50" s="3" t="inlineStr">
-        <is>
-          <t>0 de 48</t>
-        </is>
-      </c>
-      <c r="L50" s="3" t="inlineStr">
-        <is>
-          <t>0 de 48</t>
-        </is>
-      </c>
-      <c r="M50" s="3" t="inlineStr">
-        <is>
-          <t>2 de 48</t>
-        </is>
-      </c>
-      <c r="N50" s="3" t="inlineStr">
-        <is>
-          <t>0 de 48</t>
-        </is>
-      </c>
-      <c r="O50" s="3" t="inlineStr">
-        <is>
-          <t>0 de 48</t>
-        </is>
-      </c>
-      <c r="P50" s="3" t="inlineStr">
-        <is>
-          <t>0 de 48</t>
-        </is>
-      </c>
-      <c r="Q50" s="3" t="inlineStr">
-        <is>
-          <t>0 de 48</t>
-        </is>
-      </c>
-      <c r="R50" s="3" t="inlineStr">
-        <is>
-          <t>0 de 48</t>
+      <c r="C50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R50" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0 de 49</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>0 de 49</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>0 de 49</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>0 de 49</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>0 de 49</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>0 de 49</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>1 de 49</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>0 de 49</t>
+        </is>
+      </c>
+      <c r="K51" s="3" t="inlineStr">
+        <is>
+          <t>0 de 49</t>
+        </is>
+      </c>
+      <c r="L51" s="3" t="inlineStr">
+        <is>
+          <t>0 de 49</t>
+        </is>
+      </c>
+      <c r="M51" s="3" t="inlineStr">
+        <is>
+          <t>2 de 49</t>
+        </is>
+      </c>
+      <c r="N51" s="3" t="inlineStr">
+        <is>
+          <t>0 de 49</t>
+        </is>
+      </c>
+      <c r="O51" s="3" t="inlineStr">
+        <is>
+          <t>0 de 49</t>
+        </is>
+      </c>
+      <c r="P51" s="3" t="inlineStr">
+        <is>
+          <t>0 de 49</t>
+        </is>
+      </c>
+      <c r="Q51" s="3" t="inlineStr">
+        <is>
+          <t>0 de 49</t>
+        </is>
+      </c>
+      <c r="R51" s="3" t="inlineStr">
+        <is>
+          <t>0 de 49</t>
         </is>
       </c>
     </row>
@@ -3528,7 +3588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3828,7 +3888,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>COELLO TRONCOSO JOSE GREGORIO</t>
+          <t>BURNEO CELI LEYDI TATIANA</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -3855,7 +3915,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
+          <t>COELLO TRONCOSO JOSE GREGORIO</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -3882,7 +3942,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
+          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -3909,17 +3969,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
+          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>1631.15</v>
+        <v>0</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>-1206.61</v>
+        <v>0</v>
       </c>
       <c r="F14" s="2" t="n">
         <v>0</v>
@@ -3936,23 +3996,23 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
+          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0</v>
+        <v>1631.15</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0</v>
+        <v>-1206.61</v>
       </c>
       <c r="F15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -3963,7 +4023,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
+          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -3979,7 +4039,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="17">
@@ -3990,7 +4050,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
+          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -4000,7 +4060,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>1664.57</v>
+        <v>0</v>
       </c>
       <c r="F17" s="2" t="n">
         <v>0</v>
@@ -4017,17 +4077,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
+          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>4874.94</v>
+        <v>0</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0</v>
+        <v>1664.57</v>
       </c>
       <c r="F18" s="2" t="n">
         <v>0</v>
@@ -4044,14 +4104,14 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
+          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1891.36</v>
+        <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>1058.37</v>
+        <v>4874.94</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>0</v>
@@ -4060,7 +4120,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -4071,14 +4131,14 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
+          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0</v>
+        <v>1891.36</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>6342.22</v>
+        <v>1058.37</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>0</v>
@@ -4087,7 +4147,7 @@
         <v>0</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="21">
@@ -4098,14 +4158,14 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>103.71</v>
+        <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>93.98999999999999</v>
+        <v>6342.22</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>0</v>
@@ -4125,23 +4185,23 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0</v>
+        <v>103.71</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0</v>
+        <v>93.98999999999999</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>2311.23</v>
+        <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -4152,7 +4212,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>JIMENEZ GORDILLO LADY KARINA</t>
+          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -4162,13 +4222,13 @@
         <v>0</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>704.7</v>
+        <v>2311.23</v>
       </c>
       <c r="F23" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="24">
@@ -4179,17 +4239,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>JUAREZ FLORES JORGE WILLIAMS</t>
+          <t>JIMENEZ GORDILLO LADY KARINA</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1770.09</v>
+        <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>381.6</v>
+        <v>0</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0</v>
+        <v>704.7</v>
       </c>
       <c r="F24" s="2" t="n">
         <v>0</v>
@@ -4206,14 +4266,14 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>LEMA ESPINOZA MANUEL MARIA</t>
+          <t>JUAREZ FLORES JORGE WILLIAMS</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0</v>
+        <v>1770.09</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0</v>
+        <v>381.6</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>0</v>
@@ -4233,7 +4293,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>LEMA ESPINOZA MANUEL MARIA</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -4243,7 +4303,7 @@
         <v>0</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>3795.74</v>
+        <v>0</v>
       </c>
       <c r="F26" s="2" t="n">
         <v>0</v>
@@ -4260,7 +4320,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MENA COSTA GUIDO LENNIN</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -4270,7 +4330,7 @@
         <v>0</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0</v>
+        <v>3795.74</v>
       </c>
       <c r="F27" s="2" t="n">
         <v>0</v>
@@ -4287,7 +4347,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MENA COSTA GUIDO LENNIN</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -4314,7 +4374,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -4341,7 +4401,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MORALES GRACIELA ENITH</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -4351,7 +4411,7 @@
         <v>0</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>307.8</v>
+        <v>0</v>
       </c>
       <c r="F30" s="2" t="n">
         <v>0</v>
@@ -4368,7 +4428,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MORALES GRACIELA ENITH</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -4378,7 +4438,7 @@
         <v>0</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0</v>
+        <v>307.8</v>
       </c>
       <c r="F31" s="2" t="n">
         <v>0</v>
@@ -4395,14 +4455,14 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>838.7</v>
+        <v>0</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>0</v>
@@ -4422,14 +4482,14 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0</v>
+        <v>838.7</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>0</v>
@@ -4449,7 +4509,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PACHAR TAPIA ELIANA DE LOS ANGELES</t>
+          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -4476,7 +4536,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>PACHAR TAPIA ELIANA DE LOS ANGELES</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -4489,7 +4549,7 @@
         <v>0</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>153.9</v>
+        <v>0</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>0</v>
@@ -4503,7 +4563,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -4516,7 +4576,7 @@
         <v>0</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0</v>
+        <v>153.9</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>0</v>
@@ -4530,23 +4590,23 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>2179.48</v>
+        <v>0</v>
       </c>
       <c r="D37" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>744.85</v>
+        <v>0</v>
       </c>
       <c r="F37" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -4573,7 +4633,7 @@
         <v>0</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="39">
@@ -4584,23 +4644,23 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>1218.02</v>
+        <v>2179.48</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>-591.61</v>
+        <v>0</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>0</v>
+        <v>744.85</v>
       </c>
       <c r="F39" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="40">
@@ -4611,23 +4671,23 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>765.08</v>
+        <v>1218.02</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>8877.290000000001</v>
+        <v>-591.61</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>5428.56</v>
+        <v>0</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>96.37</v>
+        <v>0</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -4654,7 +4714,7 @@
         <v>96.37</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="42">
@@ -4665,23 +4725,23 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>0</v>
+        <v>765.08</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0</v>
+        <v>8877.290000000001</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0</v>
+        <v>5428.56</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0</v>
+        <v>96.37</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="43">
@@ -4692,7 +4752,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -4719,14 +4779,14 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>165.48</v>
+        <v>0</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>255.57</v>
+        <v>0</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>0</v>
@@ -4746,17 +4806,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>0</v>
+        <v>165.48</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>2963.59</v>
+        <v>255.57</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>236.11</v>
+        <v>0</v>
       </c>
       <c r="F45" s="2" t="n">
         <v>0</v>
@@ -4773,23 +4833,23 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>0</v>
+        <v>2963.59</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>3291.84</v>
+        <v>236.11</v>
       </c>
       <c r="F46" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>2500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -4816,7 +4876,7 @@
         <v>0</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>1500</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="48">
@@ -4827,7 +4887,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -4837,13 +4897,13 @@
         <v>0</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0</v>
+        <v>3291.84</v>
       </c>
       <c r="F48" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="49">
@@ -4854,17 +4914,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>SOPLIN MENDOZA TABITA</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>232.74</v>
+        <v>0</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>1489.46</v>
+        <v>0</v>
       </c>
       <c r="F49" s="2" t="n">
         <v>0</v>
@@ -4881,23 +4941,23 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>0</v>
+        <v>232.74</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>24.88</v>
+        <v>1489.46</v>
       </c>
       <c r="F50" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -4908,23 +4968,23 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>388.8</v>
+        <v>0</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>0</v>
+        <v>24.88</v>
       </c>
       <c r="F51" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="52">
@@ -4935,14 +4995,14 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>VIEJO RIVAS MAYRA ANABELLE</t>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>0</v>
+        <v>388.8</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>0</v>
@@ -4951,7 +5011,7 @@
         <v>0</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="53">
@@ -4962,39 +5022,66 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
+          <t>VIEJO RIVAS MAYRA ANABELLE</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C53" s="2" t="n">
+      <c r="C54" s="2" t="n">
         <v>1062.8</v>
       </c>
-      <c r="D53" s="2" t="n">
+      <c r="D54" s="2" t="n">
         <v>673.6900000000001</v>
       </c>
-      <c r="E53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G53" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="C54" s="4" t="n">
+      <c r="E54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="C55" s="4" t="n">
         <v>15314.18</v>
       </c>
-      <c r="D54" s="4" t="n">
+      <c r="D55" s="4" t="n">
         <v>50329.29</v>
       </c>
-      <c r="E54" s="4" t="n">
+      <c r="E55" s="4" t="n">
         <v>33603.74</v>
       </c>
-      <c r="F54" s="4" t="n">
+      <c r="F55" s="4" t="n">
         <v>461.2</v>
       </c>
-      <c r="G54" s="4" t="n">
+      <c r="G55" s="4" t="n">
         <v>24500</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-02-10 09:30:20
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -597,7 +597,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>57.28</v>
+        <v>190.94</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>0</v>
@@ -3658,7 +3658,7 @@
         <v>2444.08</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>57.28</v>
+        <v>190.94</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>2500</v>
@@ -3685,7 +3685,7 @@
         <v>2444.08</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>57.28</v>
+        <v>190.94</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>2000</v>
@@ -5079,7 +5079,7 @@
         <v>33603.74</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>461.2</v>
+        <v>728.52</v>
       </c>
       <c r="G55" s="4" t="n">
         <v>24500</v>
@@ -5104,7 +5104,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5346,13 +5346,13 @@
         <v>19250</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>153.65</v>
+        <v>287.31</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>19096.35</v>
+        <v>18962.69</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.007981818181818182</v>
+        <v>0.01492519480519481</v>
       </c>
     </row>
     <row r="11">
@@ -5389,13 +5389,13 @@
         <v>24021.08</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>307.55</v>
+        <v>441.21</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>23713.53</v>
+        <v>23579.87</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.01280333773502274</v>
+        <v>0.0183676171096387</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-10 15:30:22
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2817,7 +2817,7 @@
         <v>0</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>96.37</v>
+        <v>327.71</v>
       </c>
       <c r="N39" s="2" t="n">
         <v>0</v>
@@ -4711,7 +4711,7 @@
         <v>5428.56</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>96.37</v>
+        <v>327.71</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>2000</v>
@@ -4738,7 +4738,7 @@
         <v>5428.56</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>96.37</v>
+        <v>327.71</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>3000</v>
@@ -5079,7 +5079,7 @@
         <v>33603.74</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>1510.62</v>
+        <v>1973.3</v>
       </c>
       <c r="G55" s="4" t="n">
         <v>24500</v>
@@ -5346,13 +5346,13 @@
         <v>19250</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>287.31</v>
+        <v>518.65</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>18962.69</v>
+        <v>18731.35</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.01492519480519481</v>
+        <v>0.02694285714285714</v>
       </c>
     </row>
     <row r="11">
@@ -5389,13 +5389,13 @@
         <v>24021.08</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>1467.53</v>
+        <v>1698.87</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>22553.55</v>
+        <v>22322.21</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.06109342294351461</v>
+        <v>0.07072413063858909</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-11 17:30:19
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2802,7 +2802,7 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>0</v>
+        <v>205.2</v>
       </c>
       <c r="I39" s="2" t="n">
         <v>0</v>
@@ -3523,7 +3523,7 @@
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>2 de 49</t>
+          <t>3 de 49</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
@@ -4711,7 +4711,7 @@
         <v>5428.56</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>327.71</v>
+        <v>532.91</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>2000</v>
@@ -4738,7 +4738,7 @@
         <v>5428.56</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>327.71</v>
+        <v>532.91</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>3000</v>
@@ -5079,7 +5079,7 @@
         <v>33603.74</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>5591.95</v>
+        <v>6002.35</v>
       </c>
       <c r="G55" s="4" t="n">
         <v>24500</v>
@@ -5226,13 +5226,13 @@
         <v>560</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1397.7</v>
+        <v>1602.9</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-837.7</v>
+        <v>-1042.9</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>2.495892857142857</v>
+        <v>2.862321428571429</v>
       </c>
     </row>
     <row r="6">
@@ -5389,13 +5389,13 @@
         <v>24021.08</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>5317.52</v>
+        <v>5522.72</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>18703.56</v>
+        <v>18498.36</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.2213688976515627</v>
+        <v>0.229911394491838</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-13 16:30:22
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2817,7 +2817,7 @@
         <v>0</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>327.71</v>
+        <v>1759.79</v>
       </c>
       <c r="N39" s="2" t="n">
         <v>0</v>
@@ -4711,7 +4711,7 @@
         <v>5428.56</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>532.91</v>
+        <v>1964.99</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>2000</v>
@@ -4738,7 +4738,7 @@
         <v>5428.56</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>532.91</v>
+        <v>1964.99</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>3000</v>
@@ -5079,7 +5079,7 @@
         <v>33603.74</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>7183.01</v>
+        <v>10047.17</v>
       </c>
       <c r="G55" s="4" t="n">
         <v>24500</v>
@@ -5346,13 +5346,13 @@
         <v>19250</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>4702.36</v>
+        <v>6134.44</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>14547.64</v>
+        <v>13115.56</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.2442784415584415</v>
+        <v>0.3186722077922078</v>
       </c>
     </row>
     <row r="11">
@@ -5389,13 +5389,13 @@
         <v>24021.08</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>6703.38</v>
+        <v>8135.46</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>17317.7</v>
+        <v>15885.62</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.2790623902006071</v>
+        <v>0.3386800260437915</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-19 16:30:23
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2802,7 +2802,7 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>205.2</v>
+        <v>1333.8</v>
       </c>
       <c r="I39" s="2" t="n">
         <v>0</v>
@@ -4711,7 +4711,7 @@
         <v>5428.56</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>4829.15</v>
+        <v>5957.75</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>2000</v>
@@ -4738,7 +4738,7 @@
         <v>5428.56</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>4829.15</v>
+        <v>5957.75</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>3000</v>
@@ -5079,7 +5079,7 @@
         <v>33603.74</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>17391.55</v>
+        <v>19648.75</v>
       </c>
       <c r="G55" s="4" t="n">
         <v>24500</v>
@@ -5226,13 +5226,13 @@
         <v>560</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1602.9</v>
+        <v>2731.5</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-1042.9</v>
+        <v>-2171.5</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>2.862321428571429</v>
+        <v>4.877678571428572</v>
       </c>
     </row>
     <row r="6">
@@ -5389,13 +5389,13 @@
         <v>24021.08</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>12615.68</v>
+        <v>13744.28</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>11405.4</v>
+        <v>10276.8</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.5251920396584999</v>
+        <v>0.5721757722800139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-23 08:30:22
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2217,7 +2217,7 @@
         <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>3003.05</v>
+        <v>2981.1</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>0</v>
@@ -4474,7 +4474,7 @@
         <v>0</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>3003.05</v>
+        <v>2981.1</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>0</v>
@@ -5166,7 +5166,7 @@
         <v>33603.74</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>19648.75</v>
+        <v>19626.8</v>
       </c>
       <c r="G56" s="4" t="n">
         <v>24500</v>
@@ -5433,13 +5433,13 @@
         <v>19250</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>10614.66</v>
+        <v>10592.71</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>8635.34</v>
+        <v>8657.290000000001</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.5514109090909091</v>
+        <v>0.5502706493506493</v>
       </c>
     </row>
     <row r="11">
@@ -5476,13 +5476,13 @@
         <v>24021.08</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>13744.28</v>
+        <v>13722.33</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>10276.8</v>
+        <v>10298.75</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.5721757722800139</v>
+        <v>0.5712619915507545</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-23 16:30:23
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2097,7 +2097,7 @@
         <v>0</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>1616.06</v>
+        <v>3284.01</v>
       </c>
       <c r="N27" s="2" t="n">
         <v>0</v>
@@ -3117,7 +3117,7 @@
         <v>0</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>0</v>
+        <v>1508.82</v>
       </c>
       <c r="N44" s="2" t="n">
         <v>0</v>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="M52" s="3" t="inlineStr">
         <is>
-          <t>6 de 50</t>
+          <t>7 de 50</t>
         </is>
       </c>
       <c r="N52" s="3" t="inlineStr">
@@ -4420,7 +4420,7 @@
         <v>3795.74</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>2231.66</v>
+        <v>3899.61</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>0</v>
@@ -4933,7 +4933,7 @@
         <v>236.11</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0</v>
+        <v>1508.82</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>0</v>
@@ -5166,7 +5166,7 @@
         <v>33603.74</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>19626.8</v>
+        <v>22803.57</v>
       </c>
       <c r="G56" s="4" t="n">
         <v>24500</v>
@@ -5433,13 +5433,13 @@
         <v>19250</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>10592.71</v>
+        <v>13769.48</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>8657.290000000001</v>
+        <v>5480.52</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.5502706493506493</v>
+        <v>0.7152976623376623</v>
       </c>
     </row>
     <row r="11">
@@ -5476,13 +5476,13 @@
         <v>24021.08</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>13722.33</v>
+        <v>16899.1</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>10298.75</v>
+        <v>7121.980000000001</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.5712619915507545</v>
+        <v>0.7035112492860437</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-24 13:30:24
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -3282,7 +3282,7 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>0</v>
+        <v>782.1</v>
       </c>
       <c r="I47" s="2" t="n">
         <v>0</v>
@@ -3583,7 +3583,7 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>3 de 50</t>
+          <t>4 de 50</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
@@ -5041,7 +5041,7 @@
         <v>1489.46</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>850.1799999999999</v>
+        <v>1632.28</v>
       </c>
       <c r="G51" s="2" t="n">
         <v>0</v>
@@ -5166,7 +5166,7 @@
         <v>33603.74</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>22803.57</v>
+        <v>23585.67</v>
       </c>
       <c r="G56" s="4" t="n">
         <v>24500</v>
@@ -5313,13 +5313,13 @@
         <v>560</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>2731.5</v>
+        <v>3513.6</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-2171.5</v>
+        <v>-2953.6</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>4.877678571428572</v>
+        <v>6.274285714285714</v>
       </c>
     </row>
     <row r="6">
@@ -5476,13 +5476,13 @@
         <v>24021.08</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>16899.1</v>
+        <v>17681.2</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>7121.980000000001</v>
+        <v>6339.880000000001</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.7035112492860437</v>
+        <v>0.7360701517167421</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-25 08:30:20
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -582,7 +582,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>0</v>
+        <v>205.2</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>0</v>
@@ -597,7 +597,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>190.94</v>
+        <v>2666.92</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>0</v>
@@ -3583,7 +3583,7 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>4 de 50</t>
+          <t>5 de 50</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
@@ -3718,7 +3718,7 @@
         <v>2444.08</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>190.94</v>
+        <v>2872.12</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>2500</v>
@@ -3745,7 +3745,7 @@
         <v>2444.08</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>190.94</v>
+        <v>2872.12</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>2000</v>
@@ -5166,7 +5166,7 @@
         <v>33603.74</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>23585.67</v>
+        <v>28948.03</v>
       </c>
       <c r="G56" s="4" t="n">
         <v>24500</v>
@@ -5190,7 +5190,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5313,13 +5313,13 @@
         <v>560</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>3513.6</v>
+        <v>3718.8</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-2953.6</v>
+        <v>-3158.8</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>6.274285714285714</v>
+        <v>6.640714285714286</v>
       </c>
     </row>
     <row r="6">
@@ -5433,13 +5433,13 @@
         <v>19250</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>13769.48</v>
+        <v>16245.46</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>5480.52</v>
+        <v>3004.540000000001</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.7152976623376623</v>
+        <v>0.84392</v>
       </c>
     </row>
     <row r="11">
@@ -5476,13 +5476,13 @@
         <v>24021.08</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>17681.2</v>
+        <v>20362.38</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>6339.880000000001</v>
+        <v>3658.700000000001</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.7360701517167421</v>
+        <v>0.8476879474195164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-25 16:30:22
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -597,7 +597,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>2666.92</v>
+        <v>2770.86</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>0</v>
@@ -3718,7 +3718,7 @@
         <v>2444.08</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>2872.12</v>
+        <v>2976.06</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>2500</v>
@@ -3745,7 +3745,7 @@
         <v>2444.08</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>2872.12</v>
+        <v>2976.06</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>2000</v>
@@ -5166,7 +5166,7 @@
         <v>33603.74</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>28948.03</v>
+        <v>29155.91</v>
       </c>
       <c r="G56" s="4" t="n">
         <v>24500</v>
@@ -5189,8 +5189,8 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5433,13 +5433,13 @@
         <v>19250</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>16245.46</v>
+        <v>16349.4</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>3004.540000000001</v>
+        <v>2900.6</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.84392</v>
+        <v>0.8493194805194805</v>
       </c>
     </row>
     <row r="11">
@@ -5476,13 +5476,13 @@
         <v>24021.08</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>20362.38</v>
+        <v>20466.32</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>3658.700000000001</v>
+        <v>3554.76</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.8476879474195164</v>
+        <v>0.8520149801757456</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-26 16:30:23
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2757,7 +2757,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>0</v>
+        <v>3460.2</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>0</v>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="M52" s="3" t="inlineStr">
         <is>
-          <t>7 de 50</t>
+          <t>8 de 50</t>
         </is>
       </c>
       <c r="N52" s="3" t="inlineStr">
@@ -4717,7 +4717,7 @@
         <v>744.85</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0</v>
+        <v>3460.2</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>1500</v>
@@ -4744,7 +4744,7 @@
         <v>744.85</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0</v>
+        <v>3460.2</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>2000</v>
@@ -5166,7 +5166,7 @@
         <v>33603.74</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>29155.91</v>
+        <v>36076.31</v>
       </c>
       <c r="G56" s="4" t="n">
         <v>24500</v>
@@ -5190,7 +5190,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5433,13 +5433,13 @@
         <v>19250</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>16349.4</v>
+        <v>19809.6</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>2900.6</v>
+        <v>-559.5999999999985</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.8493194805194805</v>
+        <v>1.02907012987013</v>
       </c>
     </row>
     <row r="11">
@@ -5476,13 +5476,13 @@
         <v>24021.08</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>21747.92</v>
+        <v>25208.12</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>2273.160000000001</v>
+        <v>-1187.039999999998</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.9053681183360613</v>
+        <v>1.049416595756727</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-03 17:30:20
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -597,7 +597,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>0</v>
+        <v>1374.8</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>0</v>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="M52" s="3" t="inlineStr">
         <is>
-          <t>0 de 50</t>
+          <t>1 de 50</t>
         </is>
       </c>
       <c r="N52" s="3" t="inlineStr">
@@ -3656,7 +3656,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3718,7 +3718,7 @@
         <v>2976.06</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0</v>
+        <v>1374.8</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>2500</v>
@@ -3745,7 +3745,7 @@
         <v>2976.06</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0</v>
+        <v>1374.8</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>2000</v>
@@ -5166,7 +5166,7 @@
         <v>36208.51</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>0</v>
+        <v>2749.6</v>
       </c>
       <c r="G56" s="4" t="n">
         <v>24500</v>

</xml_diff>

<commit_message>
Actualización automática 2026-03-04 17:30:23
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -1722,7 +1722,7 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>0</v>
+        <v>782.1</v>
       </c>
       <c r="I21" s="2" t="n">
         <v>0</v>
@@ -1731,7 +1731,7 @@
         <v>0</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>0</v>
+        <v>1984.32</v>
       </c>
       <c r="L21" s="2" t="n">
         <v>0</v>
@@ -3583,22 +3583,22 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
+          <t>1 de 50</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
           <t>0 de 50</t>
         </is>
       </c>
-      <c r="I52" s="3" t="inlineStr">
+      <c r="J52" s="3" t="inlineStr">
         <is>
           <t>0 de 50</t>
         </is>
       </c>
-      <c r="J52" s="3" t="inlineStr">
-        <is>
-          <t>0 de 50</t>
-        </is>
-      </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>0 de 50</t>
+          <t>1 de 50</t>
         </is>
       </c>
       <c r="L52" s="3" t="inlineStr">
@@ -4258,7 +4258,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0</v>
+        <v>2766.42</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>0</v>
@@ -5166,7 +5166,7 @@
         <v>36208.51</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>2671.05</v>
+        <v>5437.47</v>
       </c>
       <c r="G56" s="4" t="n">
         <v>24500</v>
@@ -5313,13 +5313,13 @@
         <v>240</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0</v>
+        <v>782.1</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>240</v>
+        <v>-542.1</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0</v>
+        <v>3.25875</v>
       </c>
     </row>
     <row r="6">
@@ -5385,13 +5385,13 @@
         <v>203.76</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0</v>
+        <v>1984.32</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>203.76</v>
+        <v>-1780.56</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0</v>
+        <v>9.738515901060071</v>
       </c>
     </row>
     <row r="9">
@@ -5452,13 +5452,13 @@
         <v>47136.08</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1315.34</v>
+        <v>4081.76</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>45820.74</v>
+        <v>43054.32</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.02790516309374899</v>
+        <v>0.08659523660007365</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-05 15:30:21
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -1854,7 +1854,7 @@
         <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>0</v>
+        <v>149.26</v>
       </c>
       <c r="M23" s="2" t="n">
         <v>0</v>
@@ -3603,7 +3603,7 @@
       </c>
       <c r="L52" s="3" t="inlineStr">
         <is>
-          <t>0 de 50</t>
+          <t>1 de 50</t>
         </is>
       </c>
       <c r="M52" s="3" t="inlineStr">
@@ -4312,7 +4312,7 @@
         <v>0</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0</v>
+        <v>149.26</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>1500</v>
@@ -5166,7 +5166,7 @@
         <v>36208.51</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>5437.47</v>
+        <v>5586.73</v>
       </c>
       <c r="G56" s="4" t="n">
         <v>24500</v>
@@ -5361,10 +5361,10 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0</v>
+        <v>149.26</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0</v>
+        <v>-149.26</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0</v>
@@ -5452,13 +5452,13 @@
         <v>47136.08</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>4081.76</v>
+        <v>4231.02</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>43054.32</v>
+        <v>42905.06</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.08659523660007365</v>
+        <v>0.08976181303154612</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-09 17:30:24
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -3297,7 +3297,7 @@
         <v>0</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>0</v>
+        <v>1700.35</v>
       </c>
       <c r="N47" s="2" t="n">
         <v>0</v>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="M52" s="3" t="inlineStr">
         <is>
-          <t>2 de 50</t>
+          <t>3 de 50</t>
         </is>
       </c>
       <c r="N52" s="3" t="inlineStr">
@@ -5041,7 +5041,7 @@
         <v>1632.28</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>0</v>
+        <v>1700.35</v>
       </c>
       <c r="G51" s="2" t="n">
         <v>0</v>
@@ -5166,7 +5166,7 @@
         <v>36208.51</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>5586.73</v>
+        <v>7287.08</v>
       </c>
       <c r="G56" s="4" t="n">
         <v>24500</v>
@@ -5433,13 +5433,13 @@
         <v>43342</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>1409.33</v>
+        <v>3109.68</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>41932.67</v>
+        <v>40232.32</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.03251649670065987</v>
+        <v>0.07174749665451524</v>
       </c>
     </row>
     <row r="11">
@@ -5452,13 +5452,13 @@
         <v>47136.08</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>4231.02</v>
+        <v>5931.37</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>42905.06</v>
+        <v>41204.71</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.08976181303154612</v>
+        <v>0.1258350291326729</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-19 08:30:21
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -651,7 +651,7 @@
         <v>0</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>0</v>
+        <v>1247.9</v>
       </c>
       <c r="L3" s="2" t="n">
         <v>0</v>
@@ -3598,7 +3598,7 @@
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>1 de 50</t>
+          <t>2 de 50</t>
         </is>
       </c>
       <c r="L52" s="3" t="inlineStr">
@@ -3772,7 +3772,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0</v>
+        <v>3150.72</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>2000</v>
@@ -3826,7 +3826,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0</v>
+        <v>392.77</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>0</v>
@@ -5166,7 +5166,7 @@
         <v>36208.51</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>8144.48</v>
+        <v>11687.97</v>
       </c>
       <c r="G56" s="4" t="n">
         <v>24500</v>
@@ -5385,13 +5385,13 @@
         <v>203.76</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1984.32</v>
+        <v>3232.22</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-1780.56</v>
+        <v>-3028.46</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>9.738515901060071</v>
+        <v>15.86287789556341</v>
       </c>
     </row>
     <row r="9">
@@ -5409,13 +5409,13 @@
         <v>115</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0</v>
+        <v>2295.59</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>115</v>
+        <v>-2180.59</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0</v>
+        <v>19.96165217391304</v>
       </c>
     </row>
     <row r="10">
@@ -5452,13 +5452,13 @@
         <v>47136.08</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>6477</v>
+        <v>10020.49</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>40659.08</v>
+        <v>37115.59</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.1374106629146929</v>
+        <v>0.2125864093917016</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-19 09:30:22
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -3772,7 +3772,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>3150.72</v>
+        <v>3594.42</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>2000</v>
@@ -5166,7 +5166,7 @@
         <v>36208.51</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>11687.97</v>
+        <v>12131.67</v>
       </c>
       <c r="G56" s="4" t="n">
         <v>24500</v>
@@ -5409,13 +5409,13 @@
         <v>115</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>2295.59</v>
+        <v>2739.29</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-2180.59</v>
+        <v>-2624.29</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>19.96165217391304</v>
+        <v>23.81991304347826</v>
       </c>
     </row>
     <row r="10">
@@ -5452,13 +5452,13 @@
         <v>47136.08</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10020.49</v>
+        <v>10464.19</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>37115.59</v>
+        <v>36671.89</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.2125864093917016</v>
+        <v>0.2219995807882199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-25 12:30:18
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R52"/>
+  <dimension ref="A1:R53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
+          <t>FERRICRAFT S.A.S.</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
+          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
+          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1722,7 +1722,7 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>782.1</v>
+        <v>0</v>
       </c>
       <c r="I21" s="2" t="n">
         <v>0</v>
@@ -1731,7 +1731,7 @@
         <v>0</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>1984.32</v>
+        <v>0</v>
       </c>
       <c r="L21" s="2" t="n">
         <v>0</v>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1773,7 +1773,7 @@
         <v>0</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>-93.98999999999999</v>
+        <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
         <v>0</v>
@@ -1782,7 +1782,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>0</v>
+        <v>782.1</v>
       </c>
       <c r="I22" s="2" t="n">
         <v>0</v>
@@ -1791,7 +1791,7 @@
         <v>0</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>0</v>
+        <v>1984.32</v>
       </c>
       <c r="L22" s="2" t="n">
         <v>0</v>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1833,7 +1833,7 @@
         <v>0</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0</v>
+        <v>-93.98999999999999</v>
       </c>
       <c r="F23" s="2" t="n">
         <v>0</v>
@@ -1854,7 +1854,7 @@
         <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>149.26</v>
+        <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
         <v>0</v>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>JIMENEZ GORDILLO LADY KARINA</t>
+          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1914,7 +1914,7 @@
         <v>0</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>0</v>
+        <v>149.26</v>
       </c>
       <c r="M24" s="2" t="n">
         <v>0</v>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>JUAREZ FLORES JORGE WILLIAMS</t>
+          <t>JIMENEZ GORDILLO LADY KARINA</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -1977,7 +1977,7 @@
         <v>0</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>53.62</v>
+        <v>0</v>
       </c>
       <c r="N25" s="2" t="n">
         <v>0</v>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>LEMA ESPINOZA MANUEL MARIA</t>
+          <t>JUAREZ FLORES JORGE WILLIAMS</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2037,7 +2037,7 @@
         <v>0</v>
       </c>
       <c r="M26" s="2" t="n">
-        <v>0</v>
+        <v>53.62</v>
       </c>
       <c r="N26" s="2" t="n">
         <v>0</v>
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>LEMA ESPINOZA MANUEL MARIA</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MENA COSTA GUIDO LENNIN</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MENA COSTA GUIDO LENNIN</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MORALES GRACIELA ENITH</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MORALES GRACIELA ENITH</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PACHAR TAPIA ELIANA DE LOS ANGELES</t>
+          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>PACHAR TAPIA ELIANA DE LOS ANGELES</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2757,7 +2757,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>-90.31</v>
+        <v>0</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>0</v>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2817,7 +2817,7 @@
         <v>0</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>0</v>
+        <v>-90.31</v>
       </c>
       <c r="N39" s="2" t="n">
         <v>0</v>
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2877,7 +2877,7 @@
         <v>0</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>267.85</v>
+        <v>0</v>
       </c>
       <c r="N40" s="2" t="n">
         <v>0</v>
@@ -2886,7 +2886,7 @@
         <v>0</v>
       </c>
       <c r="P40" s="2" t="n">
-        <v>13.77</v>
+        <v>0</v>
       </c>
       <c r="Q40" s="2" t="n">
         <v>0</v>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2937,7 +2937,7 @@
         <v>0</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>0</v>
+        <v>267.85</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -2946,7 +2946,7 @@
         <v>0</v>
       </c>
       <c r="P41" s="2" t="n">
-        <v>0</v>
+        <v>13.77</v>
       </c>
       <c r="Q41" s="2" t="n">
         <v>0</v>
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>SOPLIN MENDOZA TABITA</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3297,7 +3297,7 @@
         <v>0</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>1700.35</v>
+        <v>0</v>
       </c>
       <c r="N47" s="2" t="n">
         <v>0</v>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3357,7 +3357,7 @@
         <v>0</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>0</v>
+        <v>1700.35</v>
       </c>
       <c r="N48" s="2" t="n">
         <v>0</v>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>VIEJO RIVAS MAYRA ANABELLE</t>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,137 +3503,197 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
+          <t>VIEJO RIVAS MAYRA ANABELLE</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R51" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C51" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D51" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E51" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F51" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G51" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H51" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I51" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J51" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K51" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L51" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M51" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N51" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O51" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P51" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q51" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R51" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>0 de 50</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>0 de 50</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>0 de 50</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="inlineStr">
-        <is>
-          <t>0 de 50</t>
-        </is>
-      </c>
-      <c r="G52" s="3" t="inlineStr">
-        <is>
-          <t>0 de 50</t>
-        </is>
-      </c>
-      <c r="H52" s="3" t="inlineStr">
-        <is>
-          <t>1 de 50</t>
-        </is>
-      </c>
-      <c r="I52" s="3" t="inlineStr">
-        <is>
-          <t>0 de 50</t>
-        </is>
-      </c>
-      <c r="J52" s="3" t="inlineStr">
-        <is>
-          <t>0 de 50</t>
-        </is>
-      </c>
-      <c r="K52" s="3" t="inlineStr">
-        <is>
-          <t>2 de 50</t>
-        </is>
-      </c>
-      <c r="L52" s="3" t="inlineStr">
-        <is>
-          <t>1 de 50</t>
-        </is>
-      </c>
-      <c r="M52" s="3" t="inlineStr">
-        <is>
-          <t>5 de 50</t>
-        </is>
-      </c>
-      <c r="N52" s="3" t="inlineStr">
-        <is>
-          <t>0 de 50</t>
-        </is>
-      </c>
-      <c r="O52" s="3" t="inlineStr">
-        <is>
-          <t>0 de 50</t>
-        </is>
-      </c>
-      <c r="P52" s="3" t="inlineStr">
-        <is>
-          <t>1 de 50</t>
-        </is>
-      </c>
-      <c r="Q52" s="3" t="inlineStr">
-        <is>
-          <t>0 de 50</t>
-        </is>
-      </c>
-      <c r="R52" s="3" t="inlineStr">
-        <is>
-          <t>0 de 50</t>
+      <c r="C52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R52" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0 de 51</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>0 de 51</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>0 de 51</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>0 de 51</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>0 de 51</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>1 de 51</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>0 de 51</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>0 de 51</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
+          <t>2 de 51</t>
+        </is>
+      </c>
+      <c r="L53" s="3" t="inlineStr">
+        <is>
+          <t>1 de 51</t>
+        </is>
+      </c>
+      <c r="M53" s="3" t="inlineStr">
+        <is>
+          <t>5 de 51</t>
+        </is>
+      </c>
+      <c r="N53" s="3" t="inlineStr">
+        <is>
+          <t>0 de 51</t>
+        </is>
+      </c>
+      <c r="O53" s="3" t="inlineStr">
+        <is>
+          <t>0 de 51</t>
+        </is>
+      </c>
+      <c r="P53" s="3" t="inlineStr">
+        <is>
+          <t>1 de 51</t>
+        </is>
+      </c>
+      <c r="Q53" s="3" t="inlineStr">
+        <is>
+          <t>0 de 51</t>
+        </is>
+      </c>
+      <c r="R53" s="3" t="inlineStr">
+        <is>
+          <t>0 de 51</t>
         </is>
       </c>
     </row>
@@ -3648,7 +3708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4191,11 +4251,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
+          <t>FERRICRAFT S.A.S.</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>4874.94</v>
+        <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>0</v>
@@ -4218,11 +4278,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
+          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1058.37</v>
+        <v>4874.94</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>0</v>
@@ -4234,7 +4294,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -4245,11 +4305,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
+          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>6342.22</v>
+        <v>1058.37</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>0</v>
@@ -4258,10 +4318,10 @@
         <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>2766.42</v>
+        <v>0</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="23">
@@ -4272,11 +4332,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>93.98999999999999</v>
+        <v>6342.22</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>0</v>
@@ -4285,7 +4345,7 @@
         <v>0</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>-93.98999999999999</v>
+        <v>2766.42</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>0</v>
@@ -4299,23 +4359,23 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0</v>
+        <v>93.98999999999999</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>2311.23</v>
+        <v>0</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>149.26</v>
+        <v>-93.98999999999999</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -4326,23 +4386,23 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>JIMENEZ GORDILLO LADY KARINA</t>
+          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>704.7</v>
+        <v>2311.23</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0</v>
+        <v>149.26</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="26">
@@ -4353,20 +4413,20 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>JUAREZ FLORES JORGE WILLIAMS</t>
+          <t>JIMENEZ GORDILLO LADY KARINA</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>381.6</v>
+        <v>0</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0</v>
+        <v>704.7</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>330.48</v>
+        <v>0</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>53.62</v>
+        <v>0</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>0</v>
@@ -4380,20 +4440,20 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>LEMA ESPINOZA MANUEL MARIA</t>
+          <t>JUAREZ FLORES JORGE WILLIAMS</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0</v>
+        <v>381.6</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0</v>
+        <v>330.48</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0</v>
+        <v>53.62</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>0</v>
@@ -4407,17 +4467,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>LEMA ESPINOZA MANUEL MARIA</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>3795.74</v>
+        <v>0</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>3899.61</v>
+        <v>0</v>
       </c>
       <c r="F28" s="2" t="n">
         <v>0</v>
@@ -4434,17 +4494,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MENA COSTA GUIDO LENNIN</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0</v>
+        <v>3795.74</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0</v>
+        <v>3899.61</v>
       </c>
       <c r="F29" s="2" t="n">
         <v>0</v>
@@ -4461,7 +4521,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MENA COSTA GUIDO LENNIN</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -4471,7 +4531,7 @@
         <v>0</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>2981.1</v>
+        <v>0</v>
       </c>
       <c r="F30" s="2" t="n">
         <v>0</v>
@@ -4488,7 +4548,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -4498,7 +4558,7 @@
         <v>0</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0</v>
+        <v>2981.1</v>
       </c>
       <c r="F31" s="2" t="n">
         <v>0</v>
@@ -4515,14 +4575,14 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MORALES GRACIELA ENITH</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>307.8</v>
+        <v>0</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>0</v>
@@ -4542,14 +4602,14 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MORALES GRACIELA ENITH</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0</v>
+        <v>307.8</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>0</v>
@@ -4569,17 +4629,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>838.7</v>
+        <v>0</v>
       </c>
       <c r="D34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>782.1</v>
+        <v>0</v>
       </c>
       <c r="F34" s="2" t="n">
         <v>0</v>
@@ -4596,17 +4656,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>0</v>
+        <v>838.7</v>
       </c>
       <c r="D35" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>0</v>
+        <v>782.1</v>
       </c>
       <c r="F35" s="2" t="n">
         <v>0</v>
@@ -4623,7 +4683,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PACHAR TAPIA ELIANA DE LOS ANGELES</t>
+          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -4650,7 +4710,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>PACHAR TAPIA ELIANA DE LOS ANGELES</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -4660,7 +4720,7 @@
         <v>0</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>153.9</v>
+        <v>0</v>
       </c>
       <c r="F37" s="2" t="n">
         <v>0</v>
@@ -4677,7 +4737,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -4687,7 +4747,7 @@
         <v>0</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0</v>
+        <v>153.9</v>
       </c>
       <c r="F38" s="2" t="n">
         <v>0</v>
@@ -4704,23 +4764,23 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>744.85</v>
+        <v>0</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>3460.2</v>
+        <v>0</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>-90.31</v>
+        <v>0</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -4747,7 +4807,7 @@
         <v>-90.31</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="41">
@@ -4758,23 +4818,23 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>-591.61</v>
+        <v>0</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0</v>
+        <v>744.85</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>0</v>
+        <v>3460.2</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0</v>
+        <v>-90.31</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="42">
@@ -4785,23 +4845,23 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>8877.290000000001</v>
+        <v>-591.61</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>5428.56</v>
+        <v>0</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>6023.85</v>
+        <v>0</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>281.62</v>
+        <v>0</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -4828,7 +4888,7 @@
         <v>281.62</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="44">
@@ -4839,23 +4899,23 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>0</v>
+        <v>8877.290000000001</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>0</v>
+        <v>5428.56</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>0</v>
+        <v>6023.85</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0</v>
+        <v>281.62</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="45">
@@ -4866,7 +4926,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -4893,11 +4953,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>255.57</v>
+        <v>0</v>
       </c>
       <c r="D46" s="2" t="n">
         <v>0</v>
@@ -4920,17 +4980,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>2963.59</v>
+        <v>255.57</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>236.11</v>
+        <v>0</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>1508.82</v>
+        <v>0</v>
       </c>
       <c r="F47" s="2" t="n">
         <v>0</v>
@@ -4947,23 +5007,23 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>0</v>
+        <v>2963.59</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>3291.84</v>
+        <v>236.11</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0</v>
+        <v>1508.82</v>
       </c>
       <c r="F48" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>2500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -4990,7 +5050,7 @@
         <v>0</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>1500</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="50">
@@ -5001,14 +5061,14 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>0</v>
+        <v>3291.84</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>0</v>
@@ -5017,7 +5077,7 @@
         <v>0</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="51">
@@ -5028,20 +5088,20 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>SOPLIN MENDOZA TABITA</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>232.74</v>
+        <v>0</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>1489.46</v>
+        <v>0</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>1632.28</v>
+        <v>0</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>1700.35</v>
+        <v>0</v>
       </c>
       <c r="G51" s="2" t="n">
         <v>0</v>
@@ -5055,23 +5115,23 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>0</v>
+        <v>232.74</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>24.88</v>
+        <v>1489.46</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>0</v>
+        <v>1632.28</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>0</v>
+        <v>1700.35</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -5082,14 +5142,14 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>388.8</v>
+        <v>0</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>0</v>
+        <v>24.88</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>0</v>
@@ -5098,7 +5158,7 @@
         <v>0</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="54">
@@ -5109,11 +5169,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>VIEJO RIVAS MAYRA ANABELLE</t>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>0</v>
+        <v>388.8</v>
       </c>
       <c r="D54" s="2" t="n">
         <v>0</v>
@@ -5125,7 +5185,7 @@
         <v>0</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="55">
@@ -5136,39 +5196,66 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
+          <t>VIEJO RIVAS MAYRA ANABELLE</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C55" s="2" t="n">
+      <c r="C56" s="2" t="n">
         <v>673.6900000000001</v>
       </c>
-      <c r="D55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="C56" s="4" t="n">
+      <c r="D56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="C57" s="4" t="n">
         <v>50329.29</v>
       </c>
-      <c r="D56" s="4" t="n">
+      <c r="D57" s="4" t="n">
         <v>33603.74</v>
       </c>
-      <c r="E56" s="4" t="n">
+      <c r="E57" s="4" t="n">
         <v>36208.51</v>
       </c>
-      <c r="F56" s="4" t="n">
+      <c r="F57" s="4" t="n">
         <v>12131.67</v>
       </c>
-      <c r="G56" s="4" t="n">
+      <c r="G57" s="4" t="n">
         <v>24500</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-03-27 17:30:22
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2910,7 +2910,7 @@
         <v>0</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0</v>
+        <v>763.2</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>0</v>
@@ -3623,7 +3623,7 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>0 de 51</t>
+          <t>1 de 51</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
@@ -4885,7 +4885,7 @@
         <v>6023.85</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>281.62</v>
+        <v>1044.82</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>2000</v>
@@ -4912,7 +4912,7 @@
         <v>6023.85</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>281.62</v>
+        <v>1044.82</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>3000</v>
@@ -5253,7 +5253,7 @@
         <v>36208.51</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>18448.27</v>
+        <v>19974.67</v>
       </c>
       <c r="G57" s="4" t="n">
         <v>24500</v>
@@ -5328,13 +5328,13 @@
         <v>2600</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0</v>
+        <v>763.2</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>2600</v>
+        <v>1836.8</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0</v>
+        <v>0.2935384615384616</v>
       </c>
     </row>
     <row r="3">
@@ -5539,13 +5539,13 @@
         <v>47136.08</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>16616.25</v>
+        <v>17379.45</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>30519.83</v>
+        <v>29756.63</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.3525165860207298</v>
+        <v>0.3687080045688992</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-31 09:30:19
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -3237,7 +3237,7 @@
         <v>0</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>0</v>
+        <v>17709.51</v>
       </c>
       <c r="N46" s="2" t="n">
         <v>0</v>
@@ -3668,7 +3668,7 @@
       </c>
       <c r="M53" s="3" t="inlineStr">
         <is>
-          <t>8 de 51</t>
+          <t>9 de 51</t>
         </is>
       </c>
       <c r="N53" s="3" t="inlineStr">
@@ -3716,7 +3716,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -5047,7 +5047,7 @@
         <v>0</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>0</v>
+        <v>17709.51</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>2500</v>
@@ -5074,7 +5074,7 @@
         <v>0</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>0</v>
+        <v>17709.51</v>
       </c>
       <c r="G50" s="2" t="n">
         <v>1500</v>
@@ -5253,7 +5253,7 @@
         <v>36208.51</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>25223.66</v>
+        <v>60642.68</v>
       </c>
       <c r="G57" s="4" t="n">
         <v>24500</v>
@@ -5520,13 +5520,13 @@
         <v>43342</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>13897.78</v>
+        <v>31607.29</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>29444.22</v>
+        <v>11734.71</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.3206538692261548</v>
+        <v>0.729253149370126</v>
       </c>
     </row>
     <row r="11">
@@ -5539,13 +5539,13 @@
         <v>47136.08</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>22628.44</v>
+        <v>40337.95</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>24507.64</v>
+        <v>6798.129999999999</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.4800662252779612</v>
+        <v>0.8557765092048383</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-01 13:04:34
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -3708,7 +3708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3792,17 +3792,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ALTAMIRANO ARIAS LUCIA ELIZABETH</t>
+          <t>ALTAMIRANO VILLAVICENCIO JUAN ALEJANDRO</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>2444.08</v>
+        <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2976.06</v>
+        <v>0</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>4758.49</v>
+        <v>3594.42</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>0</v>
@@ -3819,23 +3819,23 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ALTAMIRANO VILLAVICENCIO JUAN ALEJANDRO</t>
+          <t>ALVAREZ SAAVEDRA EDWIN GEOVANNY</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0</v>
+        <v>457.2</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>3594.42</v>
+        <v>0</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -3846,17 +3846,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ALVAREZ SAAVEDRA EDWIN GEOVANNY</t>
+          <t>ARMIJOS SALINAS LUIS CLAUDIO</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>457.2</v>
+        <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0</v>
+        <v>392.77</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>0</v>
@@ -3873,7 +3873,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ARMIJOS SALINAS LUIS CLAUDIO</t>
+          <t>ASES GAVILANEZ FAUSTO HERNAN</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -3883,7 +3883,7 @@
         <v>0</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>392.77</v>
+        <v>0</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>0</v>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ASES GAVILANEZ FAUSTO HERNAN</t>
+          <t>BARROS YUNGA DIEGO VINICIO</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -3927,7 +3927,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BARROS YUNGA DIEGO VINICIO</t>
+          <t>BRAVO MONTENEGRO DANIEL ANDRES</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -3954,7 +3954,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BRAVO MONTENEGRO DANIEL ANDRES</t>
+          <t>BRITO CARDENAS RUTH CECILIA</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -3981,7 +3981,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BRITO CARDENAS RUTH CECILIA</t>
+          <t>BURNEO CELI LEYDI TATIANA</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BURNEO CELI LEYDI TATIANA</t>
+          <t>COELLO TRONCOSO JOSE GREGORIO</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -4035,7 +4035,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>COELLO TRONCOSO JOSE GREGORIO</t>
+          <t>COMERCIAL AYALA VELEZ CIA LTDA</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>COMERCIAL AYALA VELEZ CIA LTDA</t>
+          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -4089,7 +4089,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
+          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -4116,11 +4116,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
+          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0</v>
+        <v>-1206.61</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>0</v>
@@ -4143,11 +4143,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
+          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-1206.61</v>
+        <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>0</v>
@@ -4159,7 +4159,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="17">
@@ -4170,7 +4170,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
+          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -4186,7 +4186,7 @@
         <v>0</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -4197,17 +4197,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
+          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0</v>
+        <v>1664.57</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0</v>
+        <v>6242.57</v>
       </c>
       <c r="F18" s="2" t="n">
         <v>0</v>
@@ -4224,17 +4224,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
+          <t>FERRICRAFT S.A.S.</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1664.57</v>
+        <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>6242.57</v>
+        <v>3120.64</v>
       </c>
       <c r="F19" s="2" t="n">
         <v>0</v>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FERRICRAFT S.A.S.</t>
+          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -4261,7 +4261,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>3120.64</v>
+        <v>0</v>
       </c>
       <c r="F20" s="2" t="n">
         <v>0</v>
@@ -4278,7 +4278,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
+          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -4294,7 +4294,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="22">
@@ -4305,7 +4305,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
+          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -4315,13 +4315,13 @@
         <v>0</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0</v>
+        <v>2766.42</v>
       </c>
       <c r="F22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -4332,7 +4332,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -4342,7 +4342,7 @@
         <v>0</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>2766.42</v>
+        <v>-93.98999999999999</v>
       </c>
       <c r="F23" s="2" t="n">
         <v>0</v>
@@ -4359,23 +4359,23 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0</v>
+        <v>2311.23</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>-93.98999999999999</v>
+        <v>149.26</v>
       </c>
       <c r="F24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="25">
@@ -4386,23 +4386,23 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
+          <t>JIMENEZ GORDILLO LADY KARINA</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>2311.23</v>
+        <v>704.7</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>149.26</v>
+        <v>0</v>
       </c>
       <c r="F25" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -4413,17 +4413,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>JIMENEZ GORDILLO LADY KARINA</t>
+          <t>JUAREZ FLORES JORGE WILLIAMS</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>704.7</v>
+        <v>0</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0</v>
+        <v>330.48</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0</v>
+        <v>53.62</v>
       </c>
       <c r="F26" s="2" t="n">
         <v>0</v>
@@ -4440,17 +4440,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>JUAREZ FLORES JORGE WILLIAMS</t>
+          <t>LEMA ESPINOZA MANUEL MARIA</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>330.48</v>
+        <v>0</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>53.62</v>
+        <v>0</v>
       </c>
       <c r="F27" s="2" t="n">
         <v>0</v>
@@ -4467,17 +4467,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>LEMA ESPINOZA MANUEL MARIA</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0</v>
+        <v>3795.74</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0</v>
+        <v>3899.61</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0</v>
+        <v>5248.3</v>
       </c>
       <c r="F28" s="2" t="n">
         <v>0</v>
@@ -4494,17 +4494,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>MENA COSTA GUIDO LENNIN</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>3795.74</v>
+        <v>0</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>3899.61</v>
+        <v>0</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>5248.3</v>
+        <v>0</v>
       </c>
       <c r="F29" s="2" t="n">
         <v>0</v>
@@ -4521,14 +4521,14 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MENA COSTA GUIDO LENNIN</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0</v>
+        <v>2981.1</v>
       </c>
       <c r="E30" s="2" t="n">
         <v>0</v>
@@ -4548,14 +4548,14 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>2981.1</v>
+        <v>0</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>0</v>
@@ -4575,17 +4575,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>MORALES GRACIELA ENITH</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0</v>
+        <v>307.8</v>
       </c>
       <c r="D32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0</v>
+        <v>367.23</v>
       </c>
       <c r="F32" s="2" t="n">
         <v>0</v>
@@ -4602,17 +4602,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MORALES GRACIELA ENITH</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>307.8</v>
+        <v>0</v>
       </c>
       <c r="D33" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>367.23</v>
+        <v>0</v>
       </c>
       <c r="F33" s="2" t="n">
         <v>0</v>
@@ -4629,14 +4629,14 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0</v>
+        <v>782.1</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>0</v>
@@ -4656,14 +4656,14 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>782.1</v>
+        <v>0</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>0</v>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
+          <t>PACHAR TAPIA ELIANA DE LOS ANGELES</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -4710,17 +4710,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PACHAR TAPIA ELIANA DE LOS ANGELES</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0</v>
+        <v>153.9</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>0</v>
+        <v>2052.08</v>
       </c>
       <c r="F37" s="2" t="n">
         <v>0</v>
@@ -4737,17 +4737,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>153.9</v>
+        <v>0</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>2052.08</v>
+        <v>0</v>
       </c>
       <c r="F38" s="2" t="n">
         <v>0</v>
@@ -4764,23 +4764,23 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>0</v>
+        <v>744.85</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0</v>
+        <v>3460.2</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>0</v>
+        <v>74.23</v>
       </c>
       <c r="F39" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="40">
@@ -4791,23 +4791,23 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>744.85</v>
+        <v>0</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>3460.2</v>
+        <v>0</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>74.23</v>
+        <v>0</v>
       </c>
       <c r="F40" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -4818,23 +4818,23 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>744.85</v>
+        <v>5428.56</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>3460.2</v>
+        <v>6023.85</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>74.23</v>
+        <v>7060.06</v>
       </c>
       <c r="F41" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="42">
@@ -4845,7 +4845,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -4872,23 +4872,23 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>5428.56</v>
+        <v>0</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>6023.85</v>
+        <v>0</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>7060.06</v>
+        <v>0</v>
       </c>
       <c r="F43" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -4899,23 +4899,23 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>5428.56</v>
+        <v>0</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>6023.85</v>
+        <v>0</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>7060.06</v>
+        <v>0</v>
       </c>
       <c r="F44" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -4926,14 +4926,14 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>0</v>
+        <v>236.11</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>0</v>
+        <v>1508.82</v>
       </c>
       <c r="E45" s="2" t="n">
         <v>0</v>
@@ -4953,23 +4953,23 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>0</v>
+        <v>3291.84</v>
       </c>
       <c r="D46" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>0</v>
+        <v>17709.51</v>
       </c>
       <c r="F46" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="47">
@@ -4980,7 +4980,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SOPLIN MENDOZA TABITA</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -5007,17 +5007,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>236.11</v>
+        <v>1489.46</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>1508.82</v>
+        <v>1632.28</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0</v>
+        <v>1700.35</v>
       </c>
       <c r="F48" s="2" t="n">
         <v>0</v>
@@ -5034,23 +5034,23 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>3291.84</v>
+        <v>24.88</v>
       </c>
       <c r="D49" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>17709.51</v>
+        <v>0</v>
       </c>
       <c r="F49" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>2500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="50">
@@ -5061,23 +5061,23 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>3291.84</v>
+        <v>0</v>
       </c>
       <c r="D50" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>17709.51</v>
+        <v>0</v>
       </c>
       <c r="F50" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="51">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>VIEJO RIVAS MAYRA ANABELLE</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -5115,17 +5115,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>1489.46</v>
+        <v>0</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>1632.28</v>
+        <v>0</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>1700.35</v>
+        <v>1635.12</v>
       </c>
       <c r="F52" s="2" t="n">
         <v>0</v>
@@ -5135,128 +5135,20 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="n">
-        <v>24.88</v>
-      </c>
-      <c r="D53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G53" s="2" t="n">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G54" s="2" t="n">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>VIEJO RIVAS MAYRA ANABELLE</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>VIVANCO MALDONADO SILVANA MARILY</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E56" s="2" t="n">
-        <v>1635.12</v>
-      </c>
-      <c r="F56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G56" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="C57" s="4" t="n">
-        <v>33603.74</v>
-      </c>
-      <c r="D57" s="4" t="n">
-        <v>36208.51</v>
-      </c>
-      <c r="E57" s="4" t="n">
-        <v>86433.37</v>
-      </c>
-      <c r="F57" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G57" s="4" t="n">
-        <v>24500</v>
+      <c r="C53" s="4" t="n">
+        <v>21694.41</v>
+      </c>
+      <c r="D53" s="4" t="n">
+        <v>23748.4</v>
+      </c>
+      <c r="E53" s="4" t="n">
+        <v>56831.08</v>
+      </c>
+      <c r="F53" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="4" t="n">
+        <v>17500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-09 15:30:19
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2937,7 +2937,7 @@
         <v>0</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>0</v>
+        <v>229.52</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -3668,7 +3668,7 @@
       </c>
       <c r="M53" s="3" t="inlineStr">
         <is>
-          <t>0 de 51</t>
+          <t>1 de 51</t>
         </is>
       </c>
       <c r="N53" s="3" t="inlineStr">
@@ -3716,7 +3716,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -4831,7 +4831,7 @@
         <v>7060.06</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0</v>
+        <v>229.52</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>3000</v>
@@ -5145,7 +5145,7 @@
         <v>56831.08</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>0</v>
+        <v>229.52</v>
       </c>
       <c r="G53" s="4" t="n">
         <v>17500</v>

</xml_diff>

<commit_message>
Actualización automática 2026-04-14 10:30:17
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2817,7 +2817,7 @@
         <v>0</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>0</v>
+        <v>5996.25</v>
       </c>
       <c r="N39" s="2" t="n">
         <v>0</v>
@@ -3668,7 +3668,7 @@
       </c>
       <c r="M53" s="3" t="inlineStr">
         <is>
-          <t>3 de 51</t>
+          <t>4 de 51</t>
         </is>
       </c>
       <c r="N53" s="3" t="inlineStr">
@@ -4777,7 +4777,7 @@
         <v>74.23</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0</v>
+        <v>5996.25</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>2000</v>
@@ -5145,7 +5145,7 @@
         <v>56831.08</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>11316.45</v>
+        <v>17312.7</v>
       </c>
       <c r="G53" s="4" t="n">
         <v>17500</v>
@@ -5168,7 +5168,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -5460,13 +5460,13 @@
         <v>26500</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>11181.45</v>
+        <v>17177.7</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>15318.55</v>
+        <v>9322.299999999999</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.4219415094339623</v>
+        <v>0.6482150943396227</v>
       </c>
     </row>
     <row r="13">
@@ -5503,13 +5503,13 @@
         <v>29134.03</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>11316.45</v>
+        <v>17312.7</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>17817.58</v>
+        <v>11821.33</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.3884272103790654</v>
+        <v>0.5942432269068165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-14 12:30:17
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2910,7 +2910,7 @@
         <v>0</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0</v>
+        <v>251.78</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>0</v>
@@ -3623,7 +3623,7 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>0 de 51</t>
+          <t>1 de 51</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
@@ -4831,7 +4831,7 @@
         <v>7060.06</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>459.04</v>
+        <v>974.11</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>3000</v>
@@ -5145,7 +5145,7 @@
         <v>56831.08</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>17312.7</v>
+        <v>17827.77</v>
       </c>
       <c r="G53" s="4" t="n">
         <v>17500</v>
@@ -5244,13 +5244,13 @@
         <v>503.71</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0</v>
+        <v>251.78</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>503.71</v>
+        <v>251.93</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0</v>
+        <v>0.4998511048023664</v>
       </c>
     </row>
     <row r="4">
@@ -5412,13 +5412,13 @@
         <v>115</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0</v>
+        <v>263.29</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>115</v>
+        <v>-148.29</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0</v>
+        <v>2.289478260869565</v>
       </c>
     </row>
     <row r="11">
@@ -5503,13 +5503,13 @@
         <v>29134.03</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>17312.7</v>
+        <v>17827.77</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>11821.33</v>
+        <v>11306.26</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.5942432269068165</v>
+        <v>0.6119225524240897</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-15 17:30:20
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -3708,7 +3708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3781,7 +3781,7 @@
         <v>0</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2500</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="3">
@@ -3808,7 +3808,7 @@
         <v>0</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -3835,7 +3835,7 @@
         <v>0</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="5">
@@ -4051,7 +4051,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="13">
@@ -4159,7 +4159,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -4213,7 +4213,7 @@
         <v>436.09</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="19">
@@ -4294,7 +4294,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -4321,7 +4321,7 @@
         <v>2192.08</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="23">
@@ -4483,7 +4483,7 @@
         <v>10149.44</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0</v>
+        <v>9500</v>
       </c>
     </row>
     <row r="29">
@@ -4737,17 +4737,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0</v>
+        <v>153.9</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0</v>
+        <v>2052.08</v>
       </c>
       <c r="F38" s="2" t="n">
         <v>0</v>
@@ -4764,23 +4764,23 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>744.85</v>
+        <v>0</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>3460.2</v>
+        <v>0</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>74.23</v>
+        <v>0</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>6128.44</v>
+        <v>0</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -4791,23 +4791,23 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>0</v>
+        <v>744.85</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0</v>
+        <v>3460.2</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>0</v>
+        <v>74.23</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0</v>
+        <v>6128.44</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="41">
@@ -4818,23 +4818,23 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>5428.56</v>
+        <v>0</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>6023.85</v>
+        <v>0</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>7060.06</v>
+        <v>0</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>974.11</v>
+        <v>0</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -4845,23 +4845,23 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>0</v>
+        <v>5428.56</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0</v>
+        <v>6023.85</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0</v>
+        <v>7060.06</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0</v>
+        <v>974.11</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="43">
@@ -4872,7 +4872,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -4899,7 +4899,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -4926,14 +4926,14 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>236.11</v>
+        <v>0</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>1508.82</v>
+        <v>0</v>
       </c>
       <c r="E45" s="2" t="n">
         <v>0</v>
@@ -4953,23 +4953,23 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>3291.84</v>
+        <v>236.11</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>0</v>
+        <v>1508.82</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>17709.51</v>
+        <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>2500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -4980,23 +4980,23 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>0</v>
+        <v>3291.84</v>
       </c>
       <c r="D47" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0</v>
+        <v>17709.51</v>
       </c>
       <c r="F47" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="48">
@@ -5007,17 +5007,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>SOPLIN MENDOZA TABITA</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>1489.46</v>
+        <v>0</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>1632.28</v>
+        <v>0</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>1700.35</v>
+        <v>0</v>
       </c>
       <c r="F48" s="2" t="n">
         <v>0</v>
@@ -5034,23 +5034,23 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>24.88</v>
+        <v>1489.46</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>0</v>
+        <v>1632.28</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>0</v>
+        <v>1700.35</v>
       </c>
       <c r="F49" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="50">
@@ -5061,11 +5061,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>0</v>
+        <v>24.88</v>
       </c>
       <c r="D50" s="2" t="n">
         <v>0</v>
@@ -5077,7 +5077,7 @@
         <v>0</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>VIEJO RIVAS MAYRA ANABELLE</t>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -5115,40 +5115,67 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
+          <t>VIEJO RIVAS MAYRA ANABELLE</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E52" s="2" t="n">
+      <c r="C53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="2" t="n">
         <v>1635.12</v>
       </c>
-      <c r="F52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G52" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="C53" s="4" t="n">
+      <c r="F53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="C54" s="4" t="n">
         <v>21694.41</v>
       </c>
-      <c r="D53" s="4" t="n">
-        <v>23748.4</v>
-      </c>
-      <c r="E53" s="4" t="n">
-        <v>56831.08</v>
-      </c>
-      <c r="F53" s="4" t="n">
+      <c r="D54" s="4" t="n">
+        <v>23902.3</v>
+      </c>
+      <c r="E54" s="4" t="n">
+        <v>58883.16</v>
+      </c>
+      <c r="F54" s="4" t="n">
         <v>19880.16</v>
       </c>
-      <c r="G53" s="4" t="n">
-        <v>17500</v>
+      <c r="G54" s="4" t="n">
+        <v>29000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-16 15:30:21
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2910,7 +2910,7 @@
         <v>0</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>251.78</v>
+        <v>587.49</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>0</v>
@@ -4858,7 +4858,7 @@
         <v>7060.06</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>899.7</v>
+        <v>1280.01</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>2000</v>
@@ -5172,7 +5172,7 @@
         <v>58883.16</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>19849.17</v>
+        <v>20229.48</v>
       </c>
       <c r="G54" s="4" t="n">
         <v>29000</v>
@@ -5196,7 +5196,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5271,13 +5271,13 @@
         <v>503.71</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>251.78</v>
+        <v>587.49</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>251.93</v>
+        <v>-83.78000000000003</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.4998511048023664</v>
+        <v>1.166325862103194</v>
       </c>
     </row>
     <row r="4">
@@ -5439,13 +5439,13 @@
         <v>115</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>263.29</v>
+        <v>307.89</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>-148.29</v>
+        <v>-192.89</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>2.289478260869565</v>
+        <v>2.677304347826087</v>
       </c>
     </row>
     <row r="11">
@@ -5530,13 +5530,13 @@
         <v>29134.03</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>19849.17</v>
+        <v>20229.48</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>9284.860000000001</v>
+        <v>8904.550000000001</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.6813053326299177</v>
+        <v>0.6943591394668023</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-21 08:30:22
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2277,7 +2277,7 @@
         <v>0</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>0</v>
+        <v>777.39</v>
       </c>
       <c r="N30" s="2" t="n">
         <v>0</v>
@@ -3668,7 +3668,7 @@
       </c>
       <c r="M53" s="3" t="inlineStr">
         <is>
-          <t>6 de 51</t>
+          <t>7 de 51</t>
         </is>
       </c>
       <c r="N53" s="3" t="inlineStr">
@@ -4534,7 +4534,7 @@
         <v>0</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0</v>
+        <v>777.39</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>0</v>
@@ -5145,7 +5145,7 @@
         <v>56831.08</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>20229.48</v>
+        <v>21006.87</v>
       </c>
       <c r="G53" s="4" t="n">
         <v>29000</v>
@@ -5168,7 +5168,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -5460,13 +5460,13 @@
         <v>26500</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>19273.51</v>
+        <v>20050.9</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>7226.490000000002</v>
+        <v>6449.099999999999</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.7273022641509433</v>
+        <v>0.7566377358490567</v>
       </c>
     </row>
     <row r="13">
@@ -5503,13 +5503,13 @@
         <v>29134.03</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>20229.48</v>
+        <v>21006.87</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>8904.550000000001</v>
+        <v>8127.16</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.6943591394668023</v>
+        <v>0.7210423686664702</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-21 14:30:21
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2277,7 +2277,7 @@
         <v>0</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>777.39</v>
+        <v>1554.78</v>
       </c>
       <c r="N30" s="2" t="n">
         <v>0</v>
@@ -4534,7 +4534,7 @@
         <v>0</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>777.39</v>
+        <v>1554.78</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>0</v>
@@ -5145,7 +5145,7 @@
         <v>56831.08</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>21006.87</v>
+        <v>21784.26</v>
       </c>
       <c r="G53" s="4" t="n">
         <v>29000</v>
@@ -5168,7 +5168,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -5460,13 +5460,13 @@
         <v>26500</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>20050.9</v>
+        <v>20828.29</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>6449.099999999999</v>
+        <v>5671.709999999999</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.7566377358490567</v>
+        <v>0.7859732075471698</v>
       </c>
     </row>
     <row r="13">
@@ -5503,13 +5503,13 @@
         <v>29134.03</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>21006.87</v>
+        <v>21784.26</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>8127.16</v>
+        <v>7349.769999999999</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.7210423686664702</v>
+        <v>0.7477255978661381</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-05-05 16:46:40
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -3781,7 +3781,7 @@
         <v>0</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>1500</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="3">
@@ -3835,7 +3835,7 @@
         <v>0</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -3862,7 +3862,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="6">
@@ -4051,7 +4051,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="13">
@@ -4078,7 +4078,7 @@
         <v>0</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>0</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="14">
@@ -4132,7 +4132,7 @@
         <v>0</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="16">
@@ -4186,7 +4186,7 @@
         <v>0</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="18">
@@ -4213,7 +4213,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="19">
@@ -4240,7 +4240,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="20">
@@ -4321,7 +4321,7 @@
         <v>0</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="23">
@@ -4375,7 +4375,7 @@
         <v>0</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="25">
@@ -4429,7 +4429,7 @@
         <v>0</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="27">
@@ -4483,7 +4483,7 @@
         <v>0</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>9500</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="29">
@@ -4537,7 +4537,7 @@
         <v>0</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="31">
@@ -4591,7 +4591,7 @@
         <v>0</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="33">
@@ -4645,7 +4645,7 @@
         <v>0</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="35">
@@ -4726,7 +4726,7 @@
         <v>0</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="38">
@@ -4780,7 +4780,7 @@
         <v>0</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="40">
@@ -4834,7 +4834,7 @@
         <v>0</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>2000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="42">
@@ -4888,7 +4888,7 @@
         <v>0</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="44">
@@ -4942,7 +4942,7 @@
         <v>0</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="46">
@@ -4969,7 +4969,7 @@
         <v>0</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>3500</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="47">
@@ -5023,7 +5023,7 @@
         <v>0</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="49">
@@ -5077,7 +5077,7 @@
         <v>0</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="51">
@@ -5131,7 +5131,7 @@
         <v>0</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="53">
@@ -5148,7 +5148,7 @@
         <v>21.71</v>
       </c>
       <c r="G53" s="4" t="n">
-        <v>29000</v>
+        <v>54500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-05-07 14:30:22
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -633,7 +633,7 @@
         <v>0</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0</v>
+        <v>93.98999999999999</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>0</v>
@@ -2937,7 +2937,7 @@
         <v>0</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>0</v>
+        <v>236.78</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -3508,47 +3508,47 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
+          <t>1 de 49</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
           <t>0 de 49</t>
         </is>
       </c>
-      <c r="F51" s="3" t="inlineStr">
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>0 de 49</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr">
         <is>
           <t>0 de 49</t>
         </is>
       </c>
-      <c r="H51" s="3" t="inlineStr">
+      <c r="I51" s="3" t="inlineStr">
         <is>
           <t>0 de 49</t>
         </is>
       </c>
-      <c r="I51" s="3" t="inlineStr">
+      <c r="J51" s="3" t="inlineStr">
         <is>
           <t>0 de 49</t>
         </is>
       </c>
-      <c r="J51" s="3" t="inlineStr">
+      <c r="K51" s="3" t="inlineStr">
         <is>
           <t>0 de 49</t>
         </is>
       </c>
-      <c r="K51" s="3" t="inlineStr">
+      <c r="L51" s="3" t="inlineStr">
         <is>
           <t>0 de 49</t>
         </is>
       </c>
-      <c r="L51" s="3" t="inlineStr">
-        <is>
-          <t>0 de 49</t>
-        </is>
-      </c>
       <c r="M51" s="3" t="inlineStr">
         <is>
-          <t>1 de 49</t>
+          <t>2 de 49</t>
         </is>
       </c>
       <c r="N51" s="3" t="inlineStr">
@@ -3596,7 +3596,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3712,7 +3712,7 @@
         <v>1814</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0</v>
+        <v>93.98999999999999</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>4000</v>
@@ -4171,7 +4171,7 @@
         <v>536.0599999999999</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0</v>
+        <v>194.22</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>1500</v>
@@ -4981,7 +4981,7 @@
         <v>93.02</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>0</v>
+        <v>236.78</v>
       </c>
       <c r="G51" s="2" t="n">
         <v>500</v>
@@ -5295,7 +5295,7 @@
         <v>36517.22</v>
       </c>
       <c r="F63" s="4" t="n">
-        <v>21.71</v>
+        <v>546.7</v>
       </c>
       <c r="G63" s="4" t="n">
         <v>54500</v>

</xml_diff>

<commit_message>
Actualización automática 2026-05-12 11:30:18
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R51"/>
+  <dimension ref="A1:R52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
+          <t>CORONEL PINOS CLARA MARIA</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1317,7 +1317,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>0</v>
+        <v>5453.44</v>
       </c>
       <c r="N14" s="2" t="n">
         <v>0</v>
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
+          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
+          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
+          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
+          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1557,7 +1557,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>35.53</v>
+        <v>0</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>FERRICRAFT S.A.S.</t>
+          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1617,7 +1617,7 @@
         <v>0</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>0</v>
+        <v>35.53</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
+          <t>FERRICRAFT S.A.S.</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
+          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
+          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>JIMENEZ GORDILLO LADY KARINA</t>
+          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>JUAREZ FLORES JORGE WILLIAMS</t>
+          <t>JIMENEZ GORDILLO LADY KARINA</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>JUAREZ FLORES JORGE WILLIAMS</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MENA COSTA GUIDO LENNIN</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MENA COSTA GUIDO LENNIN</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MORALES GRACIELA ENITH</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MORALES GRACIELA ENITH</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2577,7 +2577,7 @@
         <v>0</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>24.23</v>
+        <v>0</v>
       </c>
       <c r="N35" s="2" t="n">
         <v>0</v>
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2637,7 +2637,7 @@
         <v>0</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>0</v>
+        <v>24.23</v>
       </c>
       <c r="N36" s="2" t="n">
         <v>0</v>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2697,7 +2697,7 @@
         <v>0</v>
       </c>
       <c r="M37" s="2" t="n">
-        <v>40.93</v>
+        <v>0</v>
       </c>
       <c r="N37" s="2" t="n">
         <v>0</v>
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2757,7 +2757,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>0</v>
+        <v>40.93</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>0</v>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2937,7 +2937,7 @@
         <v>0</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>236.78</v>
+        <v>0</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -2997,7 +2997,7 @@
         <v>0</v>
       </c>
       <c r="M42" s="2" t="n">
-        <v>0</v>
+        <v>236.78</v>
       </c>
       <c r="N42" s="2" t="n">
         <v>0</v>
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>SOPLIN MENDOZA TABITA</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3357,7 +3357,7 @@
         <v>0</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>21.71</v>
+        <v>0</v>
       </c>
       <c r="N48" s="2" t="n">
         <v>0</v>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3417,7 +3417,7 @@
         <v>0</v>
       </c>
       <c r="M49" s="2" t="n">
-        <v>0</v>
+        <v>21.71</v>
       </c>
       <c r="N49" s="2" t="n">
         <v>0</v>
@@ -3443,137 +3443,197 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R50" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R50" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>0 de 49</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>0 de 49</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>1 de 49</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
-          <t>0 de 49</t>
-        </is>
-      </c>
-      <c r="G51" s="3" t="inlineStr">
-        <is>
-          <t>0 de 49</t>
-        </is>
-      </c>
-      <c r="H51" s="3" t="inlineStr">
-        <is>
-          <t>0 de 49</t>
-        </is>
-      </c>
-      <c r="I51" s="3" t="inlineStr">
-        <is>
-          <t>0 de 49</t>
-        </is>
-      </c>
-      <c r="J51" s="3" t="inlineStr">
-        <is>
-          <t>0 de 49</t>
-        </is>
-      </c>
-      <c r="K51" s="3" t="inlineStr">
-        <is>
-          <t>0 de 49</t>
-        </is>
-      </c>
-      <c r="L51" s="3" t="inlineStr">
-        <is>
-          <t>0 de 49</t>
-        </is>
-      </c>
-      <c r="M51" s="3" t="inlineStr">
-        <is>
-          <t>5 de 49</t>
-        </is>
-      </c>
-      <c r="N51" s="3" t="inlineStr">
-        <is>
-          <t>0 de 49</t>
-        </is>
-      </c>
-      <c r="O51" s="3" t="inlineStr">
-        <is>
-          <t>0 de 49</t>
-        </is>
-      </c>
-      <c r="P51" s="3" t="inlineStr">
-        <is>
-          <t>0 de 49</t>
-        </is>
-      </c>
-      <c r="Q51" s="3" t="inlineStr">
-        <is>
-          <t>0 de 49</t>
-        </is>
-      </c>
-      <c r="R51" s="3" t="inlineStr">
-        <is>
-          <t>0 de 49</t>
+      <c r="C51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R51" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0 de 50</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>0 de 50</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>1 de 50</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>0 de 50</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>0 de 50</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>0 de 50</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>0 de 50</t>
+        </is>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>0 de 50</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>0 de 50</t>
+        </is>
+      </c>
+      <c r="L52" s="3" t="inlineStr">
+        <is>
+          <t>0 de 50</t>
+        </is>
+      </c>
+      <c r="M52" s="3" t="inlineStr">
+        <is>
+          <t>6 de 50</t>
+        </is>
+      </c>
+      <c r="N52" s="3" t="inlineStr">
+        <is>
+          <t>0 de 50</t>
+        </is>
+      </c>
+      <c r="O52" s="3" t="inlineStr">
+        <is>
+          <t>0 de 50</t>
+        </is>
+      </c>
+      <c r="P52" s="3" t="inlineStr">
+        <is>
+          <t>0 de 50</t>
+        </is>
+      </c>
+      <c r="Q52" s="3" t="inlineStr">
+        <is>
+          <t>0 de 50</t>
+        </is>
+      </c>
+      <c r="R52" s="3" t="inlineStr">
+        <is>
+          <t>0 de 50</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3596,7 +3656,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -4050,7 +4110,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
+          <t>CORONEL PINOS CLARA MARIA</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -4060,13 +4120,13 @@
         <v>0</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>-1215.75</v>
+        <v>0</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>0</v>
+        <v>5453.44</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -4077,7 +4137,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
+          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -4087,13 +4147,13 @@
         <v>0</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0</v>
+        <v>-1215.75</v>
       </c>
       <c r="F18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="19">
@@ -4104,7 +4164,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ESPINOSA IDROVO RUTH CECILIA DEL CISNE</t>
+          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -4131,11 +4191,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
+          <t>ESPINOSA IDROVO RUTH CECILIA DEL CISNE</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1281.6</v>
+        <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>0</v>
@@ -4158,23 +4218,23 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
+          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0</v>
+        <v>1281.6</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>6242.57</v>
+        <v>0</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>536.0599999999999</v>
+        <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>194.22</v>
+        <v>0</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -4185,23 +4245,23 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
+          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>3015.92</v>
+        <v>6242.57</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>3767.69</v>
+        <v>536.0599999999999</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>35.53</v>
+        <v>194.22</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>3000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="23">
@@ -4212,20 +4272,20 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>FERRICRAFT S.A.S.</t>
+          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>3120.64</v>
+        <v>3015.92</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0</v>
+        <v>3767.69</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0</v>
+        <v>35.53</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>3000</v>
@@ -4239,14 +4299,14 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
+          <t>FERRICRAFT S.A.S.</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0</v>
+        <v>3120.64</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>0</v>
@@ -4255,7 +4315,7 @@
         <v>0</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="25">
@@ -4266,7 +4326,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
+          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -4293,23 +4353,23 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
+          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>2766.42</v>
+        <v>0</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>2192.08</v>
+        <v>0</v>
       </c>
       <c r="F26" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -4320,23 +4380,23 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>-93.98999999999999</v>
+        <v>2766.42</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0</v>
+        <v>2192.08</v>
       </c>
       <c r="F27" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="28">
@@ -4347,23 +4407,23 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>149.26</v>
+        <v>-93.98999999999999</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>1581.87</v>
+        <v>0</v>
       </c>
       <c r="F28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -4374,23 +4434,23 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>JARAMILLO HIDALGO DIANA ELIZABETH</t>
+          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0</v>
+        <v>149.26</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0</v>
+        <v>1581.87</v>
       </c>
       <c r="F29" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="30">
@@ -4401,7 +4461,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>JIMENEZ GORDILLO LADY KARINA</t>
+          <t>JARAMILLO HIDALGO DIANA ELIZABETH</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -4428,14 +4488,14 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>JUAREZ FLORES JORGE WILLIAMS</t>
+          <t>JIMENEZ GORDILLO LADY KARINA</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>330.48</v>
+        <v>0</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>53.62</v>
+        <v>0</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>0</v>
@@ -4444,7 +4504,7 @@
         <v>0</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -4455,14 +4515,14 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MEDINA YUNGA EDGAR VINICIO</t>
+          <t>JUAREZ FLORES JORGE WILLIAMS</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0</v>
+        <v>330.48</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0</v>
+        <v>53.62</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>0</v>
@@ -4471,7 +4531,7 @@
         <v>0</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="33">
@@ -4482,23 +4542,23 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>MEDINA YUNGA EDGAR VINICIO</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>3899.61</v>
+        <v>0</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>5248.3</v>
+        <v>0</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>10678.64</v>
+        <v>0</v>
       </c>
       <c r="F33" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>6000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -4509,23 +4569,23 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MENA COSTA GUIDO LENNIN</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0</v>
+        <v>3899.61</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0</v>
+        <v>5248.3</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>0</v>
+        <v>10678.64</v>
       </c>
       <c r="F34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>0</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="35">
@@ -4536,7 +4596,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MENA COSTA PAULA ALEJANDRA</t>
+          <t>MENA COSTA GUIDO LENNIN</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -4563,23 +4623,23 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MENA COSTA PAULA ALEJANDRA</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>2981.1</v>
+        <v>0</v>
       </c>
       <c r="D36" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>777.39</v>
+        <v>0</v>
       </c>
       <c r="F36" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -4590,23 +4650,23 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>0</v>
+        <v>2981.1</v>
       </c>
       <c r="D37" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>0</v>
+        <v>777.39</v>
       </c>
       <c r="F37" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="38">
@@ -4617,14 +4677,14 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>MORALES GRACIELA ENITH</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>367.23</v>
+        <v>0</v>
       </c>
       <c r="E38" s="2" t="n">
         <v>0</v>
@@ -4633,7 +4693,7 @@
         <v>0</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -4644,14 +4704,14 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MORALES GRACIELA ENITH</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0</v>
+        <v>367.23</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>0</v>
@@ -4660,7 +4720,7 @@
         <v>0</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="40">
@@ -4671,11 +4731,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>782.1</v>
+        <v>0</v>
       </c>
       <c r="D40" s="2" t="n">
         <v>0</v>
@@ -4687,7 +4747,7 @@
         <v>0</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -4698,11 +4758,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>0</v>
+        <v>782.1</v>
       </c>
       <c r="D41" s="2" t="n">
         <v>0</v>
@@ -4714,7 +4774,7 @@
         <v>0</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="42">
@@ -4725,7 +4785,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PALACIO ANDRADE JHONNY VICTOR</t>
+          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -4752,23 +4812,23 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>PALACIO ANDRADE JHONNY VICTOR</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>153.9</v>
+        <v>0</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>2052.08</v>
+        <v>0</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>24.23</v>
+        <v>0</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -4779,23 +4839,23 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>QUEVEDO ESPINOZA CESAR LUIS</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>0</v>
+        <v>153.9</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>0</v>
+        <v>2052.08</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0</v>
+        <v>24.23</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="45">
@@ -4806,7 +4866,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>QUEVEDO ESPINOZA CESAR LUIS</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -4833,23 +4893,23 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>3460.2</v>
+        <v>0</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>74.23</v>
+        <v>0</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>12821.43</v>
+        <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>40.93</v>
+        <v>0</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -4860,23 +4920,23 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>0</v>
+        <v>3460.2</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>0</v>
+        <v>74.23</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0</v>
+        <v>12821.43</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0</v>
+        <v>40.93</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="48">
@@ -4887,23 +4947,23 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>6023.85</v>
+        <v>0</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>7060.06</v>
+        <v>0</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>1807.7</v>
+        <v>0</v>
       </c>
       <c r="F48" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -4914,23 +4974,23 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SANCHEZ CANDO JUAN PABLO</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>0</v>
+        <v>6023.85</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>0</v>
+        <v>7060.06</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>0</v>
+        <v>1807.7</v>
       </c>
       <c r="F49" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="50">
@@ -4941,7 +5001,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+          <t>SANCHEZ CANDO JUAN PABLO</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -4968,7 +5028,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -4978,13 +5038,13 @@
         <v>0</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>93.02</v>
+        <v>0</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>236.78</v>
+        <v>0</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -4995,7 +5055,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -5005,13 +5065,13 @@
         <v>0</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>0</v>
+        <v>93.02</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>0</v>
+        <v>236.78</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="53">
@@ -5022,7 +5082,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -5049,11 +5109,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>1508.82</v>
+        <v>0</v>
       </c>
       <c r="D54" s="2" t="n">
         <v>0</v>
@@ -5065,7 +5125,7 @@
         <v>0</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -5076,14 +5136,14 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>0</v>
+        <v>1508.82</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>17709.51</v>
+        <v>0</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>0</v>
@@ -5092,7 +5152,7 @@
         <v>0</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>3000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="56">
@@ -5103,14 +5163,14 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D56" s="2" t="n">
-        <v>0</v>
+        <v>17709.51</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>0</v>
@@ -5119,7 +5179,7 @@
         <v>0</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="57">
@@ -5130,7 +5190,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>SUQUILANDA ROMA PEDRO ANDREA</t>
+          <t>SOPLIN MENDOZA TABITA</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -5157,7 +5217,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>TORRES TORRES ISABEL MERCEDES</t>
+          <t>SUQUILANDA ROMA PEDRO ANDREA</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -5184,14 +5244,14 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>TORRES TORRES ISABEL MERCEDES</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
-        <v>1632.28</v>
+        <v>0</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>1700.35</v>
+        <v>0</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>0</v>
@@ -5200,7 +5260,7 @@
         <v>0</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -5211,23 +5271,23 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
-        <v>0</v>
+        <v>1632.28</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>0</v>
+        <v>1700.35</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>43.42</v>
+        <v>0</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>21.71</v>
+        <v>0</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="61">
@@ -5238,7 +5298,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -5248,13 +5308,13 @@
         <v>0</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>0</v>
+        <v>43.42</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>0</v>
+        <v>21.71</v>
       </c>
       <c r="G61" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -5265,39 +5325,66 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C62" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D62" s="2" t="n">
+      <c r="C63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="2" t="n">
         <v>1635.12</v>
       </c>
-      <c r="E62" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F62" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G62" s="2" t="n">
+      <c r="E63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="2" t="n">
         <v>1000</v>
       </c>
     </row>
-    <row r="63">
-      <c r="C63" s="4" t="n">
+    <row r="64">
+      <c r="C64" s="4" t="n">
         <v>25274.22</v>
       </c>
-      <c r="D63" s="4" t="n">
+      <c r="D64" s="4" t="n">
         <v>59847</v>
       </c>
-      <c r="E63" s="4" t="n">
+      <c r="E64" s="4" t="n">
         <v>36517.22</v>
       </c>
-      <c r="F63" s="4" t="n">
-        <v>647.39</v>
-      </c>
-      <c r="G63" s="4" t="n">
+      <c r="F64" s="4" t="n">
+        <v>6100.83</v>
+      </c>
+      <c r="G64" s="4" t="n">
         <v>54500</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-05-12 13:30:21
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -3648,7 +3648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4920,23 +4920,23 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>REYES GUILLEN VICTOR EUGENIO</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>3460.2</v>
+        <v>0</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>74.23</v>
+        <v>0</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>12821.43</v>
+        <v>0</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>40.93</v>
+        <v>0</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -4947,23 +4947,23 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>0</v>
+        <v>3460.2</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>0</v>
+        <v>74.23</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0</v>
+        <v>12821.43</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0</v>
+        <v>40.93</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="49">
@@ -4974,23 +4974,23 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>6023.85</v>
+        <v>0</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>7060.06</v>
+        <v>0</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>1807.7</v>
+        <v>0</v>
       </c>
       <c r="F49" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -5001,23 +5001,23 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SANCHEZ CANDO JUAN PABLO</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>0</v>
+        <v>6023.85</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>0</v>
+        <v>7060.06</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>0</v>
+        <v>1807.7</v>
       </c>
       <c r="F50" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="51">
@@ -5028,7 +5028,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+          <t>SANCHEZ CANDO JUAN PABLO</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -5055,7 +5055,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -5065,13 +5065,13 @@
         <v>0</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>93.02</v>
+        <v>0</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>236.78</v>
+        <v>0</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -5082,7 +5082,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -5092,13 +5092,13 @@
         <v>0</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0</v>
+        <v>93.02</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>0</v>
+        <v>236.78</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="54">
@@ -5109,7 +5109,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -5136,11 +5136,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>1508.82</v>
+        <v>0</v>
       </c>
       <c r="D55" s="2" t="n">
         <v>0</v>
@@ -5152,7 +5152,7 @@
         <v>0</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -5163,14 +5163,14 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
-        <v>0</v>
+        <v>1508.82</v>
       </c>
       <c r="D56" s="2" t="n">
-        <v>17709.51</v>
+        <v>0</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>0</v>
@@ -5179,7 +5179,7 @@
         <v>0</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>3000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="57">
@@ -5190,14 +5190,14 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D57" s="2" t="n">
-        <v>0</v>
+        <v>17709.51</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>0</v>
@@ -5206,7 +5206,7 @@
         <v>0</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="58">
@@ -5217,7 +5217,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>SUQUILANDA ROMA PEDRO ANDREA</t>
+          <t>SOPLIN MENDOZA TABITA</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -5244,7 +5244,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>TORRES TORRES ISABEL MERCEDES</t>
+          <t>SUQUILANDA ROMA PEDRO ANDREA</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -5271,14 +5271,14 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>TORRES TORRES ISABEL MERCEDES</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
-        <v>1632.28</v>
+        <v>0</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>1700.35</v>
+        <v>0</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>0</v>
@@ -5287,7 +5287,7 @@
         <v>0</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -5298,23 +5298,23 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
-        <v>0</v>
+        <v>1632.28</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>0</v>
+        <v>1700.35</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>43.42</v>
+        <v>0</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>21.71</v>
+        <v>0</v>
       </c>
       <c r="G61" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="62">
@@ -5325,7 +5325,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -5335,13 +5335,13 @@
         <v>0</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>0</v>
+        <v>43.42</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>0</v>
+        <v>21.71</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63">
@@ -5352,39 +5352,66 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="2" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C63" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D63" s="2" t="n">
+      <c r="C64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D64" s="2" t="n">
         <v>1635.12</v>
       </c>
-      <c r="E63" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F63" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G63" s="2" t="n">
+      <c r="E64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" s="2" t="n">
         <v>1000</v>
       </c>
     </row>
-    <row r="64">
-      <c r="C64" s="4" t="n">
+    <row r="65">
+      <c r="C65" s="4" t="n">
         <v>25274.22</v>
       </c>
-      <c r="D64" s="4" t="n">
+      <c r="D65" s="4" t="n">
         <v>59847</v>
       </c>
-      <c r="E64" s="4" t="n">
+      <c r="E65" s="4" t="n">
         <v>36517.22</v>
       </c>
-      <c r="F64" s="4" t="n">
+      <c r="F65" s="4" t="n">
         <v>6100.83</v>
       </c>
-      <c r="G64" s="4" t="n">
+      <c r="G65" s="4" t="n">
         <v>54500</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-05-13 10:30:19
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -3270,7 +3270,7 @@
         <v>0</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>0</v>
+        <v>2419.77</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>0</v>
@@ -3297,7 +3297,7 @@
         <v>0</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>0</v>
+        <v>8208.35</v>
       </c>
       <c r="N47" s="2" t="n">
         <v>0</v>
@@ -3623,7 +3623,7 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>2 de 51</t>
+          <t>3 de 51</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
@@ -3668,7 +3668,7 @@
       </c>
       <c r="M53" s="3" t="inlineStr">
         <is>
-          <t>6 de 51</t>
+          <t>7 de 51</t>
         </is>
       </c>
       <c r="N53" s="3" t="inlineStr">
@@ -3716,7 +3716,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -5263,7 +5263,7 @@
         <v>0</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>0</v>
+        <v>10628.12</v>
       </c>
       <c r="G57" s="2" t="n">
         <v>3000</v>
@@ -5469,7 +5469,7 @@
         <v>36517.22</v>
       </c>
       <c r="F65" s="4" t="n">
-        <v>6520.459999999999</v>
+        <v>17148.58</v>
       </c>
       <c r="G65" s="4" t="n">
         <v>54500</v>

</xml_diff>

<commit_message>
Actualización automática 2026-05-15 12:30:18
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -3832,7 +3832,7 @@
         <v>1814</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>93.98999999999999</v>
+        <v>112.28</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>4000</v>
@@ -5469,7 +5469,7 @@
         <v>36517.22</v>
       </c>
       <c r="F65" s="4" t="n">
-        <v>17148.58</v>
+        <v>17166.87</v>
       </c>
       <c r="G65" s="4" t="n">
         <v>54500</v>

</xml_diff>

<commit_message>
Actualización automática 2026-06-01 15:30:20
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -657,7 +657,7 @@
         <v>0</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>0</v>
+        <v>16.2</v>
       </c>
       <c r="N3" s="2" t="n">
         <v>0</v>
@@ -3728,7 +3728,7 @@
       </c>
       <c r="M54" s="3" t="inlineStr">
         <is>
-          <t>0 de 52</t>
+          <t>1 de 52</t>
         </is>
       </c>
       <c r="N54" s="3" t="inlineStr">
@@ -3892,7 +3892,7 @@
         <v>37.09</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0</v>
+        <v>16.2</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>4000</v>
@@ -5556,7 +5556,7 @@
         <v>40247.96</v>
       </c>
       <c r="F66" s="4" t="n">
-        <v>0</v>
+        <v>16.2</v>
       </c>
       <c r="G66" s="4" t="n">
         <v>56500</v>

</xml_diff>

<commit_message>
Actualización automática 2026-06-10 14:30:22
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2970,7 +2970,7 @@
         <v>0</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0</v>
+        <v>191.07</v>
       </c>
       <c r="E42" s="2" t="n">
         <v>0</v>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>1 de 52</t>
+          <t>2 de 52</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
@@ -5188,7 +5188,7 @@
         <v>1219.26</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>6152.78</v>
+        <v>6343.85</v>
       </c>
       <c r="G52" s="2" t="n">
         <v>8000</v>
@@ -5583,7 +5583,7 @@
         <v>43159.64</v>
       </c>
       <c r="F67" s="4" t="n">
-        <v>9698.07</v>
+        <v>9889.140000000001</v>
       </c>
       <c r="G67" s="4" t="n">
         <v>44000</v>

</xml_diff>

<commit_message>
Actualización automática 2026-06-19 12:30:19
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -1557,7 +1557,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>0</v>
+        <v>3072.2</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -3848,7 +3848,7 @@
       </c>
       <c r="M56" s="3" t="inlineStr">
         <is>
-          <t>7 de 54</t>
+          <t>8 de 54</t>
         </is>
       </c>
       <c r="N56" s="3" t="inlineStr">
@@ -4498,7 +4498,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0</v>
+        <v>3072.2</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>0</v>
@@ -5730,7 +5730,7 @@
         <v>40247.96</v>
       </c>
       <c r="F68" s="4" t="n">
-        <v>20497.97</v>
+        <v>23570.17</v>
       </c>
       <c r="G68" s="4" t="n">
         <v>0</v>
@@ -5997,13 +5997,13 @@
         <v>39858</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>17850.14</v>
+        <v>20922.34</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>22007.86</v>
+        <v>18935.66</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.4478433438707411</v>
+        <v>0.5249219730041648</v>
       </c>
     </row>
     <row r="11">
@@ -6040,13 +6040,13 @@
         <v>44641.5</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>20497.97</v>
+        <v>23570.17</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>24143.53</v>
+        <v>21071.33</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.4591684867219963</v>
+        <v>0.5279878588309084</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-22 17:30:18
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R56"/>
+  <dimension ref="A1:R57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3597,7 +3597,7 @@
         <v>0</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>0</v>
+        <v>4237.6</v>
       </c>
       <c r="N52" s="2" t="n">
         <v>0</v>
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,137 +3743,197 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R55" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R55" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>2 de 54</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="F56" s="3" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="H56" s="3" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="I56" s="3" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="J56" s="3" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="K56" s="3" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="L56" s="3" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="M56" s="3" t="inlineStr">
-        <is>
-          <t>9 de 54</t>
-        </is>
-      </c>
-      <c r="N56" s="3" t="inlineStr">
-        <is>
-          <t>1 de 54</t>
-        </is>
-      </c>
-      <c r="O56" s="3" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="P56" s="3" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="Q56" s="3" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
-        </is>
-      </c>
-      <c r="R56" s="3" t="inlineStr">
-        <is>
-          <t>0 de 54</t>
+      <c r="C56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R56" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>2 de 55</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="L57" s="3" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="M57" s="3" t="inlineStr">
+        <is>
+          <t>10 de 55</t>
+        </is>
+      </c>
+      <c r="N57" s="3" t="inlineStr">
+        <is>
+          <t>1 de 55</t>
+        </is>
+      </c>
+      <c r="O57" s="3" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="P57" s="3" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="Q57" s="3" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
+        </is>
+      </c>
+      <c r="R57" s="3" t="inlineStr">
+        <is>
+          <t>0 de 55</t>
         </is>
       </c>
     </row>
@@ -3888,7 +3948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5592,7 +5652,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>TORRES TORRES ISABEL MERCEDES</t>
+          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -5605,7 +5665,7 @@
         <v>0</v>
       </c>
       <c r="F63" s="2" t="n">
-        <v>0</v>
+        <v>4237.6</v>
       </c>
       <c r="G63" s="2" t="n">
         <v>0</v>
@@ -5619,11 +5679,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>TORRES TORRES ISABEL MERCEDES</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
-        <v>1700.35</v>
+        <v>0</v>
       </c>
       <c r="D64" s="2" t="n">
         <v>0</v>
@@ -5646,17 +5706,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
-        <v>0</v>
+        <v>1700.35</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>43.42</v>
+        <v>0</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>21.71</v>
+        <v>0</v>
       </c>
       <c r="F65" s="2" t="n">
         <v>0</v>
@@ -5673,17 +5733,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>0</v>
+        <v>43.42</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>0</v>
+        <v>21.71</v>
       </c>
       <c r="F66" s="2" t="n">
         <v>0</v>
@@ -5700,39 +5760,66 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C67" s="2" t="n">
+      <c r="C68" s="2" t="n">
         <v>1635.12</v>
       </c>
-      <c r="D67" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E67" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F67" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G67" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="C68" s="4" t="n">
+      <c r="D68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="C69" s="4" t="n">
         <v>59847</v>
       </c>
-      <c r="D68" s="4" t="n">
+      <c r="D69" s="4" t="n">
         <v>36517.22</v>
       </c>
-      <c r="E68" s="4" t="n">
+      <c r="E69" s="4" t="n">
         <v>40247.96</v>
       </c>
-      <c r="F68" s="4" t="n">
-        <v>25787.35</v>
-      </c>
-      <c r="G68" s="4" t="n">
+      <c r="F69" s="4" t="n">
+        <v>30024.95</v>
+      </c>
+      <c r="G69" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5997,13 +6084,13 @@
         <v>39858</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>23074.73</v>
+        <v>27312.33</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>16783.27</v>
+        <v>12545.67</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.5789234281700035</v>
+        <v>0.6852408550353756</v>
       </c>
     </row>
     <row r="11">
@@ -6040,13 +6127,13 @@
         <v>44641.5</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>25787.35</v>
+        <v>30024.95</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>18854.15</v>
+        <v>14616.55</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.5776542006877009</v>
+        <v>0.672579326411523</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-23 16:30:21
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -657,7 +657,7 @@
         <v>0</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>1442.45</v>
+        <v>3889.77</v>
       </c>
       <c r="N3" s="2" t="n">
         <v>0</v>
@@ -3117,7 +3117,7 @@
         <v>0</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>7046.23</v>
+        <v>7197.82</v>
       </c>
       <c r="N44" s="2" t="n">
         <v>114.3</v>
@@ -4072,7 +4072,7 @@
         <v>37.09</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1626.45</v>
+        <v>4073.77</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>0</v>
@@ -5395,7 +5395,7 @@
         <v>1219.26</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>7955.89</v>
+        <v>8107.48</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>0</v>
@@ -5817,7 +5817,7 @@
         <v>40247.96</v>
       </c>
       <c r="F69" s="4" t="n">
-        <v>30019.37</v>
+        <v>32618.28</v>
       </c>
       <c r="G69" s="4" t="n">
         <v>0</v>
@@ -6084,13 +6084,13 @@
         <v>39858</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>27306.75</v>
+        <v>29905.66</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>12551.25</v>
+        <v>9952.34</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.6851008580460636</v>
+        <v>0.750305083044809</v>
       </c>
     </row>
     <row r="11">
@@ -6127,13 +6127,13 @@
         <v>44641.5</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>30019.37</v>
+        <v>32618.28</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>14622.13</v>
+        <v>12023.22</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.6724543306116506</v>
+        <v>0.7306716844192063</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-09 16:30:16
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -3126,7 +3126,7 @@
         <v>0</v>
       </c>
       <c r="P44" s="2" t="n">
-        <v>0</v>
+        <v>55.06</v>
       </c>
       <c r="Q44" s="2" t="n">
         <v>0</v>
@@ -3923,7 +3923,7 @@
       </c>
       <c r="P57" s="3" t="inlineStr">
         <is>
-          <t>0 de 55</t>
+          <t>1 de 55</t>
         </is>
       </c>
       <c r="Q57" s="3" t="inlineStr">
@@ -5098,7 +5098,7 @@
         <v>9109.299999999999</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0</v>
+        <v>134.36</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>0</v>
@@ -5412,7 +5412,7 @@
         <v>35603.86</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>426.67</v>
+        <v>561.03</v>
       </c>
       <c r="G54" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-07-10 14:30:16
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R57"/>
+  <dimension ref="A1:R58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
+          <t>CARRION MORALES CARLOS ENRIQUE</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -1197,7 +1197,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>0</v>
+        <v>50.54</v>
       </c>
       <c r="N12" s="2" t="n">
         <v>0</v>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
+          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CORONEL PINOS CLARA MARIA</t>
+          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
+          <t>CORONEL PINOS CLARA MARIA</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
+          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
+          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
+          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1557,7 +1557,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>426.67</v>
+        <v>0</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
+          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1617,7 +1617,7 @@
         <v>0</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>0</v>
+        <v>426.67</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
+          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FERRICRAFT S.A.S.</t>
+          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
+          <t>FERRICRAFT S.A.S.</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GLOBAL MOYANO &amp; ASOCIADOS LEMO S.A.S.</t>
+          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
+          <t>GLOBAL MOYANO &amp; ASOCIADOS LEMO S.A.S.</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
+          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>JIMENEZ GORDILLO LADY KARINA</t>
+          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>JUAREZ FLORES JORGE WILLIAMS</t>
+          <t>JIMENEZ GORDILLO LADY KARINA</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>LEMA ESPINOZA MANUEL MARIA</t>
+          <t>JUAREZ FLORES JORGE WILLIAMS</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>LEMA ESPINOZA MANUEL MARIA</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MENA COSTA GUIDO LENNIN</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MENA COSTA GUIDO LENNIN</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MORALES GRACIELA ENITH</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MORALES GRACIELA ENITH</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>REYES GUILLEN VICTOR EUGENIO</t>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>REYES GUILLEN VICTOR EUGENIO</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3126,7 +3126,7 @@
         <v>0</v>
       </c>
       <c r="P44" s="2" t="n">
-        <v>55.06</v>
+        <v>0</v>
       </c>
       <c r="Q44" s="2" t="n">
         <v>0</v>
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3186,7 +3186,7 @@
         <v>0</v>
       </c>
       <c r="P45" s="2" t="n">
-        <v>0</v>
+        <v>55.06</v>
       </c>
       <c r="Q45" s="2" t="n">
         <v>0</v>
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
+          <t>SOPLIN MENDOZA TABITA</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,137 +3803,197 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R56" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R56" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="F57" s="3" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="G57" s="3" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="H57" s="3" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="I57" s="3" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="J57" s="3" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="K57" s="3" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="L57" s="3" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="M57" s="3" t="inlineStr">
-        <is>
-          <t>1 de 55</t>
-        </is>
-      </c>
-      <c r="N57" s="3" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="O57" s="3" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="P57" s="3" t="inlineStr">
-        <is>
-          <t>1 de 55</t>
-        </is>
-      </c>
-      <c r="Q57" s="3" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
-        </is>
-      </c>
-      <c r="R57" s="3" t="inlineStr">
-        <is>
-          <t>0 de 55</t>
+      <c r="C57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R57" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="L58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="M58" s="3" t="inlineStr">
+        <is>
+          <t>2 de 56</t>
+        </is>
+      </c>
+      <c r="N58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="O58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="P58" s="3" t="inlineStr">
+        <is>
+          <t>1 de 56</t>
+        </is>
+      </c>
+      <c r="Q58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="R58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
         </is>
       </c>
     </row>
@@ -3948,7 +4008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4302,7 +4362,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
+          <t>CARRION MORALES CARLOS ENRIQUE</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -4315,7 +4375,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0</v>
+        <v>50.54</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>0</v>
@@ -4329,7 +4389,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
+          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -4356,14 +4416,14 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CORONEL PINOS CLARA MARIA</t>
+          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>9255.389999999999</v>
+        <v>0</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>0</v>
@@ -4383,14 +4443,14 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
+          <t>CORONEL PINOS CLARA MARIA</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-1215.75</v>
+        <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0</v>
+        <v>9255.389999999999</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>0</v>
@@ -4410,11 +4470,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
+          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0</v>
+        <v>-1215.75</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>0</v>
@@ -4437,14 +4497,14 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
+          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>1089.28</v>
+        <v>0</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>0</v>
@@ -4464,20 +4524,20 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
+          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0</v>
+        <v>1089.28</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>3072.2</v>
+        <v>0</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>426.67</v>
+        <v>0</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>0</v>
@@ -4491,20 +4551,20 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
+          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>536.0599999999999</v>
+        <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>187.92</v>
+        <v>0</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0</v>
+        <v>3072.2</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0</v>
+        <v>426.67</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>0</v>
@@ -4518,17 +4578,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
+          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>3767.69</v>
+        <v>536.0599999999999</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>35.53</v>
+        <v>187.92</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>4096.36</v>
+        <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
         <v>0</v>
@@ -4545,17 +4605,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
+          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0</v>
+        <v>3767.69</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0</v>
+        <v>35.53</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0</v>
+        <v>4096.36</v>
       </c>
       <c r="F22" s="2" t="n">
         <v>0</v>
@@ -4572,7 +4632,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GLOBAL MOYANO &amp; ASOCIADOS LEMO S.A.S.</t>
+          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -4582,7 +4642,7 @@
         <v>0</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>70.37</v>
+        <v>0</v>
       </c>
       <c r="F23" s="2" t="n">
         <v>0</v>
@@ -4599,7 +4659,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
+          <t>GLOBAL MOYANO &amp; ASOCIADOS LEMO S.A.S.</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -4609,7 +4669,7 @@
         <v>0</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0</v>
+        <v>70.37</v>
       </c>
       <c r="F24" s="2" t="n">
         <v>0</v>
@@ -4626,17 +4686,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
+          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>2192.08</v>
+        <v>0</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>4922.83</v>
+        <v>0</v>
       </c>
       <c r="F25" s="2" t="n">
         <v>0</v>
@@ -4653,17 +4713,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
+          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1581.87</v>
+        <v>2192.08</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0</v>
+        <v>4922.83</v>
       </c>
       <c r="F26" s="2" t="n">
         <v>0</v>
@@ -4680,11 +4740,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>JIMENEZ GORDILLO LADY KARINA</t>
+          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0</v>
+        <v>1581.87</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>0</v>
@@ -4707,7 +4767,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>JUAREZ FLORES JORGE WILLIAMS</t>
+          <t>JIMENEZ GORDILLO LADY KARINA</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -4734,7 +4794,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>LEMA ESPINOZA MANUEL MARIA</t>
+          <t>JUAREZ FLORES JORGE WILLIAMS</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -4744,7 +4804,7 @@
         <v>0</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>865.47</v>
+        <v>0</v>
       </c>
       <c r="F29" s="2" t="n">
         <v>0</v>
@@ -4761,17 +4821,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>LEMA ESPINOZA MANUEL MARIA</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>10678.64</v>
+        <v>0</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>10260.43</v>
+        <v>0</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0</v>
+        <v>865.47</v>
       </c>
       <c r="F30" s="2" t="n">
         <v>0</v>
@@ -4788,14 +4848,14 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MENA COSTA GUIDO LENNIN</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0</v>
+        <v>10678.64</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0</v>
+        <v>10260.43</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>0</v>
@@ -4815,11 +4875,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MENA COSTA GUIDO LENNIN</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>777.39</v>
+        <v>0</v>
       </c>
       <c r="D32" s="2" t="n">
         <v>0</v>
@@ -4842,11 +4902,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>0</v>
+        <v>777.39</v>
       </c>
       <c r="D33" s="2" t="n">
         <v>0</v>
@@ -4869,14 +4929,14 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MORALES GRACIELA ENITH</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>986.58</v>
+        <v>0</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>0</v>
@@ -4896,17 +4956,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MORALES GRACIELA ENITH</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0</v>
+        <v>986.58</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>16.74</v>
+        <v>0</v>
       </c>
       <c r="F35" s="2" t="n">
         <v>0</v>
@@ -4923,7 +4983,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -4933,7 +4993,7 @@
         <v>0</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0</v>
+        <v>16.74</v>
       </c>
       <c r="F36" s="2" t="n">
         <v>0</v>
@@ -4950,14 +5010,14 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>2911.68</v>
+        <v>0</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>0</v>
@@ -4977,14 +5037,14 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0</v>
+        <v>2911.68</v>
       </c>
       <c r="E38" s="2" t="n">
         <v>0</v>
@@ -5004,17 +5064,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>REYES GUILLEN VICTOR EUGENIO</t>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>167.85</v>
+        <v>0</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>1882.6</v>
+        <v>0</v>
       </c>
       <c r="F39" s="2" t="n">
         <v>0</v>
@@ -5031,17 +5091,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>REYES GUILLEN VICTOR EUGENIO</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>12821.43</v>
+        <v>0</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>292.71</v>
+        <v>167.85</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>101.16</v>
+        <v>1882.6</v>
       </c>
       <c r="F40" s="2" t="n">
         <v>0</v>
@@ -5058,17 +5118,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>0</v>
+        <v>12821.43</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0</v>
+        <v>292.71</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>0</v>
+        <v>101.16</v>
       </c>
       <c r="F41" s="2" t="n">
         <v>0</v>
@@ -5085,20 +5145,20 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>1807.7</v>
+        <v>0</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>1219.26</v>
+        <v>0</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>9109.299999999999</v>
+        <v>0</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>134.36</v>
+        <v>0</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>0</v>
@@ -5112,20 +5172,20 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>0</v>
+        <v>1807.7</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>0</v>
+        <v>1219.26</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0</v>
+        <v>9109.299999999999</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0</v>
+        <v>134.36</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>0</v>
@@ -5139,14 +5199,14 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>93.02</v>
+        <v>0</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>236.78</v>
+        <v>0</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>0</v>
@@ -5166,14 +5226,14 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>0</v>
+        <v>93.02</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>0</v>
+        <v>236.78</v>
       </c>
       <c r="E45" s="2" t="n">
         <v>0</v>
@@ -5193,14 +5253,14 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>2917.63</v>
+        <v>0</v>
       </c>
       <c r="E46" s="2" t="n">
         <v>0</v>
@@ -5220,17 +5280,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>10628.12</v>
+        <v>2917.63</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>3155.46</v>
+        <v>0</v>
       </c>
       <c r="F47" s="2" t="n">
         <v>0</v>
@@ -5247,17 +5307,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>0</v>
+        <v>10628.12</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0</v>
+        <v>3155.46</v>
       </c>
       <c r="F48" s="2" t="n">
         <v>0</v>
@@ -5274,7 +5334,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
+          <t>SOPLIN MENDOZA TABITA</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -5284,7 +5344,7 @@
         <v>0</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>4237.6</v>
+        <v>0</v>
       </c>
       <c r="F49" s="2" t="n">
         <v>0</v>
@@ -5301,7 +5361,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -5311,7 +5371,7 @@
         <v>0</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>0</v>
+        <v>4237.6</v>
       </c>
       <c r="F50" s="2" t="n">
         <v>0</v>
@@ -5328,14 +5388,14 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>43.42</v>
+        <v>0</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>21.71</v>
+        <v>0</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>0</v>
@@ -5355,14 +5415,14 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>0</v>
+        <v>43.42</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>0</v>
+        <v>21.71</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>0</v>
@@ -5382,39 +5442,66 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G53" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="C54" s="4" t="n">
+      <c r="C54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="C55" s="4" t="n">
         <v>36517.22</v>
       </c>
-      <c r="D54" s="4" t="n">
+      <c r="D55" s="4" t="n">
         <v>40247.96</v>
       </c>
-      <c r="E54" s="4" t="n">
+      <c r="E55" s="4" t="n">
         <v>35603.86</v>
       </c>
-      <c r="F54" s="4" t="n">
-        <v>561.03</v>
-      </c>
-      <c r="G54" s="4" t="n">
+      <c r="F55" s="4" t="n">
+        <v>611.5700000000001</v>
+      </c>
+      <c r="G55" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-07-14 11:30:15
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -810,7 +810,7 @@
         <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0</v>
+        <v>1049.69</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>0</v>
@@ -3923,7 +3923,7 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>0 de 56</t>
+          <t>1 de 56</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
@@ -4016,7 +4016,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -4213,7 +4213,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0</v>
+        <v>1049.69</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>0</v>
@@ -5499,7 +5499,7 @@
         <v>35603.86</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>611.5700000000001</v>
+        <v>1661.26</v>
       </c>
       <c r="G55" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-07-14 14:30:15
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -3273,7 +3273,7 @@
         <v>0</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0</v>
+        <v>148.54</v>
       </c>
       <c r="F47" s="2" t="n">
         <v>0</v>
@@ -3928,7 +3928,7 @@
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>0 de 56</t>
+          <t>1 de 56</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
@@ -5239,7 +5239,7 @@
         <v>0</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0</v>
+        <v>148.54</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>0</v>
@@ -5499,7 +5499,7 @@
         <v>35603.86</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>1661.26</v>
+        <v>1809.8</v>
       </c>
       <c r="G55" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-07-21 08:30:17
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -633,31 +633,31 @@
         <v>0</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0</v>
+        <v>548.78</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0</v>
+        <v>391.37</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>0</v>
+        <v>230.47</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>0</v>
+        <v>199.36</v>
       </c>
       <c r="L3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>0</v>
+        <v>6.32</v>
       </c>
       <c r="N3" s="2" t="n">
         <v>0</v>
@@ -1986,7 +1986,7 @@
         <v>0</v>
       </c>
       <c r="P25" s="2" t="n">
-        <v>0</v>
+        <v>702.0599999999999</v>
       </c>
       <c r="Q25" s="2" t="n">
         <v>0</v>
@@ -2154,7 +2154,7 @@
         <v>0</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>0</v>
+        <v>522.55</v>
       </c>
       <c r="M28" s="2" t="n">
         <v>0</v>
@@ -3177,7 +3177,7 @@
         <v>0</v>
       </c>
       <c r="M45" s="2" t="n">
-        <v>0</v>
+        <v>4462.17</v>
       </c>
       <c r="N45" s="2" t="n">
         <v>0</v>
@@ -3928,62 +3928,62 @@
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
+          <t>2 de 56</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
           <t>1 de 56</t>
         </is>
       </c>
-      <c r="F58" s="3" t="inlineStr">
+      <c r="H58" s="3" t="inlineStr">
         <is>
           <t>0 de 56</t>
         </is>
       </c>
-      <c r="G58" s="3" t="inlineStr">
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>1 de 56</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
         <is>
           <t>0 de 56</t>
         </is>
       </c>
-      <c r="H58" s="3" t="inlineStr">
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>1 de 56</t>
+        </is>
+      </c>
+      <c r="L58" s="3" t="inlineStr">
+        <is>
+          <t>1 de 56</t>
+        </is>
+      </c>
+      <c r="M58" s="3" t="inlineStr">
+        <is>
+          <t>5 de 56</t>
+        </is>
+      </c>
+      <c r="N58" s="3" t="inlineStr">
         <is>
           <t>0 de 56</t>
         </is>
       </c>
-      <c r="I58" s="3" t="inlineStr">
+      <c r="O58" s="3" t="inlineStr">
         <is>
           <t>0 de 56</t>
         </is>
       </c>
-      <c r="J58" s="3" t="inlineStr">
-        <is>
-          <t>0 de 56</t>
-        </is>
-      </c>
-      <c r="K58" s="3" t="inlineStr">
-        <is>
-          <t>0 de 56</t>
-        </is>
-      </c>
-      <c r="L58" s="3" t="inlineStr">
-        <is>
-          <t>0 de 56</t>
-        </is>
-      </c>
-      <c r="M58" s="3" t="inlineStr">
-        <is>
-          <t>3 de 56</t>
-        </is>
-      </c>
-      <c r="N58" s="3" t="inlineStr">
-        <is>
-          <t>0 de 56</t>
-        </is>
-      </c>
-      <c r="O58" s="3" t="inlineStr">
-        <is>
-          <t>0 de 56</t>
-        </is>
-      </c>
       <c r="P58" s="3" t="inlineStr">
         <is>
-          <t>1 de 56</t>
+          <t>2 de 56</t>
         </is>
       </c>
       <c r="Q58" s="3" t="inlineStr">
@@ -4105,7 +4105,7 @@
         <v>4073.77</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0</v>
+        <v>1513.66</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>0</v>
@@ -4699,7 +4699,7 @@
         <v>0</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>343.7</v>
+        <v>1045.76</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>0</v>
@@ -4753,7 +4753,7 @@
         <v>0</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0</v>
+        <v>522.55</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>0</v>
@@ -5185,7 +5185,7 @@
         <v>9109.299999999999</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>372.25</v>
+        <v>4834.42</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>0</v>
@@ -5499,7 +5499,7 @@
         <v>35603.86</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>2391.39</v>
+        <v>9591.83</v>
       </c>
       <c r="G55" s="4" t="n">
         <v>0</v>
@@ -5523,7 +5523,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5598,13 +5598,13 @@
         <v>199.5</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>148.54</v>
+        <v>697.3200000000001</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>50.96000000000001</v>
+        <v>-497.8200000000001</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.7445614035087719</v>
+        <v>3.495338345864662</v>
       </c>
     </row>
     <row r="4">
@@ -5622,13 +5622,13 @@
         <v>172.82</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0</v>
+        <v>391.37</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>172.82</v>
+        <v>-218.55</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0</v>
+        <v>2.264610577479459</v>
       </c>
     </row>
     <row r="5">
@@ -5646,13 +5646,13 @@
         <v>263</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0</v>
+        <v>230.47</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>263</v>
+        <v>32.53</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0</v>
+        <v>0.8763117870722433</v>
       </c>
     </row>
     <row r="6">
@@ -5670,10 +5670,10 @@
         <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>55.06</v>
+        <v>1279.67</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-55.06</v>
+        <v>-1279.67</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0</v>
@@ -5694,13 +5694,13 @@
         <v>203.76</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0</v>
+        <v>199.36</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>203.76</v>
+        <v>4.399999999999977</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0</v>
+        <v>0.9784059678052612</v>
       </c>
     </row>
     <row r="8">
@@ -5718,13 +5718,13 @@
         <v>115</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>317.19</v>
+        <v>454.55</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-202.19</v>
+        <v>-339.55</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>2.758173913043478</v>
+        <v>3.952608695652174</v>
       </c>
     </row>
     <row r="9">
@@ -5742,13 +5742,13 @@
         <v>35342</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>820.91</v>
+        <v>5289.4</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>34521.09</v>
+        <v>30052.6</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.0232276045498274</v>
+        <v>0.1496632901363816</v>
       </c>
     </row>
     <row r="10">
@@ -5761,13 +5761,13 @@
         <v>38896.08</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>2391.39</v>
+        <v>9591.83</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>36504.69</v>
+        <v>29304.25</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.06148151690350287</v>
+        <v>0.2466014570105779</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-21 16:30:19
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -897,7 +897,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>0</v>
+        <v>1284.32</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -1377,7 +1377,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>0</v>
+        <v>2068.01</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -3510,7 +3510,7 @@
         <v>0</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>0</v>
+        <v>1348.76</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>0</v>
@@ -3923,52 +3923,52 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
+          <t>2 de 56</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>2 de 56</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
           <t>1 de 56</t>
         </is>
       </c>
-      <c r="E58" s="3" t="inlineStr">
-        <is>
-          <t>2 de 56</t>
-        </is>
-      </c>
-      <c r="F58" s="3" t="inlineStr">
+      <c r="H58" s="3" t="inlineStr">
         <is>
           <t>0 de 56</t>
         </is>
       </c>
-      <c r="G58" s="3" t="inlineStr">
+      <c r="I58" s="3" t="inlineStr">
         <is>
           <t>1 de 56</t>
         </is>
       </c>
-      <c r="H58" s="3" t="inlineStr">
+      <c r="J58" s="3" t="inlineStr">
         <is>
           <t>0 de 56</t>
         </is>
       </c>
-      <c r="I58" s="3" t="inlineStr">
+      <c r="K58" s="3" t="inlineStr">
         <is>
           <t>1 de 56</t>
         </is>
       </c>
-      <c r="J58" s="3" t="inlineStr">
-        <is>
-          <t>0 de 56</t>
-        </is>
-      </c>
-      <c r="K58" s="3" t="inlineStr">
+      <c r="L58" s="3" t="inlineStr">
         <is>
           <t>1 de 56</t>
         </is>
       </c>
-      <c r="L58" s="3" t="inlineStr">
-        <is>
-          <t>1 de 56</t>
-        </is>
-      </c>
       <c r="M58" s="3" t="inlineStr">
         <is>
-          <t>6 de 56</t>
+          <t>8 de 56</t>
         </is>
       </c>
       <c r="N58" s="3" t="inlineStr">
@@ -4240,7 +4240,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0</v>
+        <v>1284.32</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>0</v>
@@ -4456,7 +4456,7 @@
         <v>0</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0</v>
+        <v>2068.01</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>0</v>
@@ -5320,7 +5320,7 @@
         <v>3155.46</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0</v>
+        <v>1348.76</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>0</v>
@@ -5499,7 +5499,7 @@
         <v>35603.86</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>9626.130000000001</v>
+        <v>14327.22</v>
       </c>
       <c r="G55" s="4" t="n">
         <v>0</v>
@@ -5574,13 +5574,13 @@
         <v>2600</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1049.69</v>
+        <v>2398.45</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1550.31</v>
+        <v>201.5500000000002</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.4037269230769231</v>
+        <v>0.9224807692307692</v>
       </c>
     </row>
     <row r="3">
@@ -5742,13 +5742,13 @@
         <v>35342</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>5323.7</v>
+        <v>8676.030000000001</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>30018.3</v>
+        <v>26665.97</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.1506338068021051</v>
+        <v>0.2454878048780488</v>
       </c>
     </row>
     <row r="10">
@@ -5761,13 +5761,13 @@
         <v>38896.08</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>9626.130000000001</v>
+        <v>14327.22</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>29269.95</v>
+        <v>24568.86</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.2474832939463308</v>
+        <v>0.368346116112472</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-22 08:30:20
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2154,7 +2154,7 @@
         <v>0</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>522.55</v>
+        <v>1479.64</v>
       </c>
       <c r="M28" s="2" t="n">
         <v>0</v>
@@ -4753,7 +4753,7 @@
         <v>0</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>522.55</v>
+        <v>1479.64</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>0</v>
@@ -5499,7 +5499,7 @@
         <v>35603.86</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>14327.22</v>
+        <v>15284.31</v>
       </c>
       <c r="G55" s="4" t="n">
         <v>0</v>
@@ -5670,10 +5670,10 @@
         <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1279.67</v>
+        <v>2236.76</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-1279.67</v>
+        <v>-2236.76</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0</v>
@@ -5761,13 +5761,13 @@
         <v>38896.08</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>14327.22</v>
+        <v>15284.31</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>24568.86</v>
+        <v>23611.77</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.368346116112472</v>
+        <v>0.3929524517637767</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-27 08:30:20
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R59"/>
+  <dimension ref="A1:R58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -563,7 +563,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AGUILAR OROZCO SANTOS EULIDIO</t>
+          <t>ALTAMIRANO ARIAS LUCIA ELIZABETH</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -573,31 +573,31 @@
         <v>0</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0</v>
+        <v>548.78</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0</v>
+        <v>391.37</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>0</v>
+        <v>230.47</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>0</v>
+        <v>199.36</v>
       </c>
       <c r="L2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>0</v>
+        <v>6.32</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>0</v>
@@ -623,7 +623,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ALTAMIRANO ARIAS LUCIA ELIZABETH</t>
+          <t>ALTAMIRANO VILLAVICENCIO JUAN ALEJANDRO</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -633,31 +633,31 @@
         <v>0</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>548.78</v>
+        <v>0</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>391.37</v>
+        <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>230.47</v>
+        <v>0</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>199.36</v>
+        <v>0</v>
       </c>
       <c r="L3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>6.32</v>
+        <v>0</v>
       </c>
       <c r="N3" s="2" t="n">
         <v>0</v>
@@ -683,7 +683,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ALTAMIRANO VILLAVICENCIO JUAN ALEJANDRO</t>
+          <t>ALVAREZ SAAVEDRA EDWIN GEOVANNY</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -743,14 +743,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ALVAREZ SAAVEDRA EDWIN GEOVANNY</t>
+          <t>ARIAS CARDENAS BOLIVAR MAURICIO</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0</v>
+        <v>1049.69</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0</v>
@@ -803,14 +803,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ARIAS CARDENAS BOLIVAR MAURICIO</t>
+          <t>ARMIJOS SALINAS LUIS CLAUDIO</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1049.69</v>
+        <v>0</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>0</v>
@@ -837,7 +837,7 @@
         <v>0</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>0</v>
+        <v>1284.32</v>
       </c>
       <c r="N6" s="2" t="n">
         <v>0</v>
@@ -863,7 +863,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ARMIJOS SALINAS LUIS CLAUDIO</t>
+          <t>ASES GAVILANEZ FAUSTO HERNAN</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -897,7 +897,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>1284.32</v>
+        <v>0</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -923,7 +923,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ASES GAVILANEZ FAUSTO HERNAN</t>
+          <t>BARROS YUNGA DIEGO VINICIO</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BARROS YUNGA DIEGO VINICIO</t>
+          <t>BRAVO MONTENEGRO DANIEL ANDRES</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BRAVO MONTENEGRO DANIEL ANDRES</t>
+          <t>BRITO CARDENAS RUTH CECILIA</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BRITO CARDENAS RUTH CECILIA</t>
+          <t>CARRION MORALES CARLOS ENRIQUE</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -1137,7 +1137,7 @@
         <v>0</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>0</v>
+        <v>50.54</v>
       </c>
       <c r="N11" s="2" t="n">
         <v>0</v>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CARRION MORALES CARLOS ENRIQUE</t>
+          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -1197,7 +1197,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>50.54</v>
+        <v>0</v>
       </c>
       <c r="N12" s="2" t="n">
         <v>0</v>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
+          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
+          <t>CORONEL PINOS CLARA MARIA</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1317,7 +1317,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>0</v>
+        <v>2068.01</v>
       </c>
       <c r="N14" s="2" t="n">
         <v>0</v>
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CORONEL PINOS CLARA MARIA</t>
+          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1377,7 +1377,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>2068.01</v>
+        <v>0</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
+          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
+          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
+          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1557,7 +1557,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>0</v>
+        <v>426.67</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
+          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1617,7 +1617,7 @@
         <v>0</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>426.67</v>
+        <v>34.3</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
+          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1677,7 +1677,7 @@
         <v>0</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>34.3</v>
+        <v>0</v>
       </c>
       <c r="N20" s="2" t="n">
         <v>0</v>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
+          <t>FERRICRAFT S.A.S.</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>FERRICRAFT S.A.S.</t>
+          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
+          <t>GLOBAL MOYANO &amp; ASOCIADOS LEMO S.A.S.</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>GLOBAL MOYANO &amp; ASOCIADOS LEMO S.A.S.</t>
+          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1917,7 +1917,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>0</v>
+        <v>343.7</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -1926,7 +1926,7 @@
         <v>0</v>
       </c>
       <c r="P24" s="2" t="n">
-        <v>0</v>
+        <v>702.0599999999999</v>
       </c>
       <c r="Q24" s="2" t="n">
         <v>0</v>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
+          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -1977,7 +1977,7 @@
         <v>0</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>343.7</v>
+        <v>0</v>
       </c>
       <c r="N25" s="2" t="n">
         <v>0</v>
@@ -1986,7 +1986,7 @@
         <v>0</v>
       </c>
       <c r="P25" s="2" t="n">
-        <v>702.0599999999999</v>
+        <v>0</v>
       </c>
       <c r="Q25" s="2" t="n">
         <v>0</v>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2094,7 +2094,7 @@
         <v>0</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>0</v>
+        <v>1479.64</v>
       </c>
       <c r="M27" s="2" t="n">
         <v>0</v>
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
+          <t>JIMENEZ GORDILLO LADY KARINA</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2154,7 +2154,7 @@
         <v>0</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>1479.64</v>
+        <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
         <v>0</v>
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>JIMENEZ GORDILLO LADY KARINA</t>
+          <t>JUAREZ FLORES JORGE WILLIAMS</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>JUAREZ FLORES JORGE WILLIAMS</t>
+          <t>LEMA ESPINOZA MANUEL MARIA</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>LEMA ESPINOZA MANUEL MARIA</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>MENA COSTA GUIDO LENNIN</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MENA COSTA GUIDO LENNIN</t>
+          <t>MENESES TORRES OSCAR LEONARDO</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2451,7 +2451,7 @@
         <v>0</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>0</v>
+        <v>401.57</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>0</v>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MENESES TORRES OSCAR LEONARDO</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2511,7 +2511,7 @@
         <v>0</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>401.57</v>
+        <v>0</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>0</v>
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>MORALES GRACIELA ENITH</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MORALES GRACIELA ENITH</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2877,7 +2877,7 @@
         <v>0</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>0</v>
+        <v>321.93</v>
       </c>
       <c r="N40" s="2" t="n">
         <v>0</v>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2937,7 +2937,7 @@
         <v>0</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>321.93</v>
+        <v>0</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>REYES GUILLEN VICTOR EUGENIO</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>REYES GUILLEN VICTOR EUGENIO</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3177,7 +3177,7 @@
         <v>0</v>
       </c>
       <c r="M45" s="2" t="n">
-        <v>0</v>
+        <v>4462.17</v>
       </c>
       <c r="N45" s="2" t="n">
         <v>0</v>
@@ -3186,7 +3186,7 @@
         <v>0</v>
       </c>
       <c r="P45" s="2" t="n">
-        <v>0</v>
+        <v>55.06</v>
       </c>
       <c r="Q45" s="2" t="n">
         <v>0</v>
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3237,7 +3237,7 @@
         <v>0</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>4462.17</v>
+        <v>0</v>
       </c>
       <c r="N46" s="2" t="n">
         <v>0</v>
@@ -3246,7 +3246,7 @@
         <v>0</v>
       </c>
       <c r="P46" s="2" t="n">
-        <v>55.06</v>
+        <v>0</v>
       </c>
       <c r="Q46" s="2" t="n">
         <v>0</v>
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3273,7 +3273,7 @@
         <v>0</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0</v>
+        <v>148.54</v>
       </c>
       <c r="F47" s="2" t="n">
         <v>0</v>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3333,7 +3333,7 @@
         <v>0</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>148.54</v>
+        <v>0</v>
       </c>
       <c r="F48" s="2" t="n">
         <v>0</v>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,14 +3503,14 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>0</v>
+        <v>1348.76</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>0</v>
@@ -3563,14 +3563,14 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>SOPLIN MENDOZA TABITA</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>1348.76</v>
+        <v>0</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>0</v>
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3916,144 +3916,84 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>VIVANCO MALDONADO SILVANA MARILY</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R58" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>2 de 57</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr">
-        <is>
-          <t>2 de 57</t>
-        </is>
-      </c>
-      <c r="F59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="G59" s="3" t="inlineStr">
-        <is>
-          <t>1 de 57</t>
-        </is>
-      </c>
-      <c r="H59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="I59" s="3" t="inlineStr">
-        <is>
-          <t>1 de 57</t>
-        </is>
-      </c>
-      <c r="J59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="K59" s="3" t="inlineStr">
-        <is>
-          <t>2 de 57</t>
-        </is>
-      </c>
-      <c r="L59" s="3" t="inlineStr">
-        <is>
-          <t>1 de 57</t>
-        </is>
-      </c>
-      <c r="M59" s="3" t="inlineStr">
-        <is>
-          <t>9 de 57</t>
-        </is>
-      </c>
-      <c r="N59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="O59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="P59" s="3" t="inlineStr">
-        <is>
-          <t>2 de 57</t>
-        </is>
-      </c>
-      <c r="Q59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="R59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>2 de 56</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>2 de 56</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>1 de 56</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>1 de 56</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>2 de 56</t>
+        </is>
+      </c>
+      <c r="L58" s="3" t="inlineStr">
+        <is>
+          <t>1 de 56</t>
+        </is>
+      </c>
+      <c r="M58" s="3" t="inlineStr">
+        <is>
+          <t>9 de 56</t>
+        </is>
+      </c>
+      <c r="N58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="O58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="P58" s="3" t="inlineStr">
+        <is>
+          <t>2 de 56</t>
+        </is>
+      </c>
+      <c r="Q58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="R58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-08-03 11:30:16
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -1317,7 +1317,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>0</v>
+        <v>708.88</v>
       </c>
       <c r="N14" s="2" t="n">
         <v>0</v>
@@ -4028,7 +4028,7 @@
       </c>
       <c r="M59" s="3" t="inlineStr">
         <is>
-          <t>0 de 57</t>
+          <t>1 de 57</t>
         </is>
       </c>
       <c r="N59" s="3" t="inlineStr">
@@ -4516,7 +4516,7 @@
         <v>2068.01</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0</v>
+        <v>708.88</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>0</v>
@@ -5613,7 +5613,7 @@
         <v>28143.93</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>0</v>
+        <v>708.88</v>
       </c>
       <c r="G57" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-08-03 16:30:17
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -3090,7 +3090,7 @@
         <v>0</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>0</v>
+        <v>706.3099999999999</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>0</v>
@@ -3597,7 +3597,7 @@
         <v>0</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>0</v>
+        <v>1925.42</v>
       </c>
       <c r="N52" s="2" t="n">
         <v>0</v>
@@ -3983,52 +3983,52 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
+          <t>1 de 57</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
           <t>0 de 57</t>
         </is>
       </c>
-      <c r="E59" s="3" t="inlineStr">
+      <c r="F59" s="3" t="inlineStr">
         <is>
           <t>0 de 57</t>
         </is>
       </c>
-      <c r="F59" s="3" t="inlineStr">
+      <c r="G59" s="3" t="inlineStr">
         <is>
           <t>0 de 57</t>
         </is>
       </c>
-      <c r="G59" s="3" t="inlineStr">
+      <c r="H59" s="3" t="inlineStr">
         <is>
           <t>0 de 57</t>
         </is>
       </c>
-      <c r="H59" s="3" t="inlineStr">
+      <c r="I59" s="3" t="inlineStr">
         <is>
           <t>0 de 57</t>
         </is>
       </c>
-      <c r="I59" s="3" t="inlineStr">
+      <c r="J59" s="3" t="inlineStr">
         <is>
           <t>0 de 57</t>
         </is>
       </c>
-      <c r="J59" s="3" t="inlineStr">
+      <c r="K59" s="3" t="inlineStr">
         <is>
           <t>0 de 57</t>
         </is>
       </c>
-      <c r="K59" s="3" t="inlineStr">
+      <c r="L59" s="3" t="inlineStr">
         <is>
           <t>0 de 57</t>
         </is>
       </c>
-      <c r="L59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
       <c r="M59" s="3" t="inlineStr">
         <is>
-          <t>1 de 57</t>
+          <t>2 de 57</t>
         </is>
       </c>
       <c r="N59" s="3" t="inlineStr">
@@ -4076,7 +4076,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -5245,7 +5245,7 @@
         <v>2180.13</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0</v>
+        <v>706.3099999999999</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>0</v>
@@ -5434,7 +5434,7 @@
         <v>1348.76</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>0</v>
+        <v>1925.42</v>
       </c>
       <c r="G50" s="2" t="n">
         <v>0</v>
@@ -5613,7 +5613,7 @@
         <v>28143.93</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>708.88</v>
+        <v>3340.61</v>
       </c>
       <c r="G57" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-08-05 12:30:17
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2097,7 +2097,7 @@
         <v>0</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>0</v>
+        <v>2451.41</v>
       </c>
       <c r="N27" s="2" t="n">
         <v>0</v>
@@ -4028,7 +4028,7 @@
       </c>
       <c r="M59" s="3" t="inlineStr">
         <is>
-          <t>3 de 57</t>
+          <t>4 de 57</t>
         </is>
       </c>
       <c r="N59" s="3" t="inlineStr">
@@ -4813,7 +4813,7 @@
         <v>1479.64</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0</v>
+        <v>2451.41</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>0</v>
@@ -5613,7 +5613,7 @@
         <v>28143.93</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>4890.85</v>
+        <v>7342.26</v>
       </c>
       <c r="G57" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-08-07 17:30:15
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2094,7 +2094,7 @@
         <v>0</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>0</v>
+        <v>261.27</v>
       </c>
       <c r="M27" s="2" t="n">
         <v>2451.41</v>
@@ -4023,7 +4023,7 @@
       </c>
       <c r="L59" s="3" t="inlineStr">
         <is>
-          <t>0 de 57</t>
+          <t>1 de 57</t>
         </is>
       </c>
       <c r="M59" s="3" t="inlineStr">
@@ -4813,7 +4813,7 @@
         <v>1479.64</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>2451.41</v>
+        <v>2712.68</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>0</v>
@@ -5613,7 +5613,7 @@
         <v>28143.93</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>8475.83</v>
+        <v>8737.1</v>
       </c>
       <c r="G57" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-08-12 08:30:18
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -1137,7 +1137,7 @@
         <v>0</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>0</v>
+        <v>258.49</v>
       </c>
       <c r="N11" s="2" t="n">
         <v>0</v>
@@ -4028,7 +4028,7 @@
       </c>
       <c r="M59" s="3" t="inlineStr">
         <is>
-          <t>5 de 57</t>
+          <t>6 de 57</t>
         </is>
       </c>
       <c r="N59" s="3" t="inlineStr">
@@ -4435,7 +4435,7 @@
         <v>50.54</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0</v>
+        <v>258.49</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>0</v>
@@ -5613,7 +5613,7 @@
         <v>28143.93</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>8737.1</v>
+        <v>8995.59</v>
       </c>
       <c r="G57" s="4" t="n">
         <v>0</v>
@@ -5904,13 +5904,13 @@
         <v>35342</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>7769.52</v>
+        <v>8028.01</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>27572.48</v>
+        <v>27313.99</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.219838152905891</v>
+        <v>0.2271521136325052</v>
       </c>
     </row>
     <row r="12">
@@ -5923,13 +5923,13 @@
         <v>40778.76</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>8737.1</v>
+        <v>8995.59</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>32041.66</v>
+        <v>31783.17</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.2142561470726427</v>
+        <v>0.2205949862134111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-12 16:30:18
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -3477,7 +3477,7 @@
         <v>0</v>
       </c>
       <c r="M50" s="2" t="n">
-        <v>0</v>
+        <v>474.08</v>
       </c>
       <c r="N50" s="2" t="n">
         <v>0</v>
@@ -4028,7 +4028,7 @@
       </c>
       <c r="M59" s="3" t="inlineStr">
         <is>
-          <t>6 de 57</t>
+          <t>7 de 57</t>
         </is>
       </c>
       <c r="N59" s="3" t="inlineStr">
@@ -5380,7 +5380,7 @@
         <v>0</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0</v>
+        <v>474.08</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>0</v>
@@ -5613,7 +5613,7 @@
         <v>28143.93</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>8995.59</v>
+        <v>9469.67</v>
       </c>
       <c r="G57" s="4" t="n">
         <v>0</v>
@@ -5904,13 +5904,13 @@
         <v>35342</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>8028.01</v>
+        <v>8502.09</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>27313.99</v>
+        <v>26839.91</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.2271521136325052</v>
+        <v>0.2405661818799162</v>
       </c>
     </row>
     <row r="12">
@@ -5923,13 +5923,13 @@
         <v>40778.76</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>8995.59</v>
+        <v>9469.67</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>31783.17</v>
+        <v>31309.09</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.2205949862134111</v>
+        <v>0.2322206462383849</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-18 08:30:18
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -1317,7 +1317,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>708.88</v>
+        <v>3169.83</v>
       </c>
       <c r="N14" s="2" t="n">
         <v>0</v>
@@ -3597,7 +3597,7 @@
         <v>0</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>1925.42</v>
+        <v>13692.06</v>
       </c>
       <c r="N52" s="2" t="n">
         <v>0</v>
@@ -4076,7 +4076,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -4516,7 +4516,7 @@
         <v>2068.01</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>708.88</v>
+        <v>3169.83</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>0</v>
@@ -5434,7 +5434,7 @@
         <v>1348.76</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>1925.42</v>
+        <v>13692.06</v>
       </c>
       <c r="G50" s="2" t="n">
         <v>0</v>
@@ -5613,7 +5613,7 @@
         <v>28143.93</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>14053.12</v>
+        <v>28280.71</v>
       </c>
       <c r="G57" s="4" t="n">
         <v>0</v>
@@ -5637,7 +5637,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5904,13 +5904,13 @@
         <v>35342</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>13085.54</v>
+        <v>27313.13</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>22256.46</v>
+        <v>8028.869999999999</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.370254654518703</v>
+        <v>0.7728235527134854</v>
       </c>
     </row>
     <row r="12">
@@ -5923,13 +5923,13 @@
         <v>40778.76</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>14053.12</v>
+        <v>28280.71</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>26725.64</v>
+        <v>12498.05</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.3446186200855543</v>
+        <v>0.6935156929734989</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-19 09:30:18
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2094,7 +2094,7 @@
         <v>0</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>261.27</v>
+        <v>0</v>
       </c>
       <c r="M27" s="2" t="n">
         <v>2451.41</v>
@@ -3357,7 +3357,7 @@
         <v>0</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>0</v>
+        <v>-1284.32</v>
       </c>
       <c r="N48" s="2" t="n">
         <v>0</v>
@@ -4023,7 +4023,7 @@
       </c>
       <c r="L59" s="3" t="inlineStr">
         <is>
-          <t>1 de 57</t>
+          <t>0 de 57</t>
         </is>
       </c>
       <c r="M59" s="3" t="inlineStr">
@@ -4813,7 +4813,7 @@
         <v>1479.64</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>2712.68</v>
+        <v>2451.41</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>0</v>
@@ -5353,7 +5353,7 @@
         <v>1432.86</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0</v>
+        <v>-1284.32</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>0</v>
@@ -5613,7 +5613,7 @@
         <v>28143.93</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>28280.71</v>
+        <v>26735.12</v>
       </c>
       <c r="G57" s="4" t="n">
         <v>0</v>
@@ -5880,13 +5880,13 @@
         <v>960</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>261.27</v>
+        <v>0</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>698.73</v>
+        <v>960</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.27215625</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -5904,13 +5904,13 @@
         <v>35342</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>27313.13</v>
+        <v>26028.81</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>8028.869999999999</v>
+        <v>9313.189999999999</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.7728235527134854</v>
+        <v>0.7364837869956427</v>
       </c>
     </row>
     <row r="12">
@@ -5923,13 +5923,13 @@
         <v>40778.76</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>28280.71</v>
+        <v>26735.12</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>12498.05</v>
+        <v>14043.64</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.6935156929734989</v>
+        <v>0.6556138538788331</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-21 10:30:18
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -1317,7 +1317,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>3169.83</v>
+        <v>5446.06</v>
       </c>
       <c r="N14" s="2" t="n">
         <v>0</v>
@@ -3117,7 +3117,7 @@
         <v>0</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>0</v>
+        <v>1640.63</v>
       </c>
       <c r="N44" s="2" t="n">
         <v>0</v>
@@ -4028,7 +4028,7 @@
       </c>
       <c r="M59" s="3" t="inlineStr">
         <is>
-          <t>9 de 57</t>
+          <t>10 de 57</t>
         </is>
       </c>
       <c r="N59" s="3" t="inlineStr">
@@ -4516,7 +4516,7 @@
         <v>2068.01</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>3169.83</v>
+        <v>5446.06</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>0</v>
@@ -5245,7 +5245,7 @@
         <v>2180.13</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>706.3099999999999</v>
+        <v>2346.94</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>0</v>
@@ -5613,7 +5613,7 @@
         <v>28143.93</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>27897.35</v>
+        <v>31814.21</v>
       </c>
       <c r="G57" s="4" t="n">
         <v>0</v>
@@ -5636,7 +5636,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -5904,13 +5904,13 @@
         <v>35342</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>26097.04</v>
+        <v>30013.9</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>9244.959999999999</v>
+        <v>5328.099999999999</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.7384143511968763</v>
+        <v>0.8492416954331957</v>
       </c>
     </row>
     <row r="12">
@@ -5923,13 +5923,13 @@
         <v>40778.76</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>27897.35</v>
+        <v>31814.21</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>12881.41</v>
+        <v>8964.549999999999</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.6841147205064597</v>
+        <v>0.7801661943619669</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-25 16:30:19
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -3117,7 +3117,7 @@
         <v>0</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>1640.63</v>
+        <v>2379.4</v>
       </c>
       <c r="N44" s="2" t="n">
         <v>0</v>
@@ -5245,7 +5245,7 @@
         <v>2180.13</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>2346.94</v>
+        <v>3085.71</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>0</v>
@@ -5613,7 +5613,7 @@
         <v>28143.93</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>31814.21</v>
+        <v>32552.98</v>
       </c>
       <c r="G57" s="4" t="n">
         <v>0</v>
@@ -5636,7 +5636,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -5904,13 +5904,13 @@
         <v>35342</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>30013.9</v>
+        <v>30752.67</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>5328.099999999999</v>
+        <v>4589.330000000002</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.8492416954331957</v>
+        <v>0.8701451530756606</v>
       </c>
     </row>
     <row r="12">
@@ -5923,13 +5923,13 @@
         <v>40778.76</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>31814.21</v>
+        <v>32552.98</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>8964.549999999999</v>
+        <v>8225.780000000002</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.7801661943619669</v>
+        <v>0.7982827334622239</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-28 16:30:19
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -1971,7 +1971,7 @@
         <v>0</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>0</v>
+        <v>1499.16</v>
       </c>
       <c r="L25" s="2" t="n">
         <v>0</v>
@@ -4018,7 +4018,7 @@
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>1 de 57</t>
+          <t>2 de 57</t>
         </is>
       </c>
       <c r="L59" s="3" t="inlineStr">
@@ -4786,7 +4786,7 @@
         <v>0</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0</v>
+        <v>1499.16</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>0</v>
@@ -5613,7 +5613,7 @@
         <v>28143.93</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>42034.27</v>
+        <v>43533.43</v>
       </c>
       <c r="G57" s="4" t="n">
         <v>0</v>
@@ -5808,13 +5808,13 @@
         <v>203.76</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>369.92</v>
+        <v>1869.08</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-166.16</v>
+        <v>-1665.32</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>1.815469179426777</v>
+        <v>9.1729485669415</v>
       </c>
     </row>
     <row r="8">
@@ -5899,13 +5899,13 @@
         <v>40081.76</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>42034.27</v>
+        <v>43533.43</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-1952.509999999999</v>
+        <v>-3451.669999999999</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>1.048713180259549</v>
+        <v>1.086115729449006</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-04 12:30:14
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -4068,7 +4068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5205,23 +5205,23 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0</v>
+        <v>1432.86</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0</v>
+        <v>-1284.32</v>
       </c>
       <c r="F42" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="43">
@@ -5232,23 +5232,23 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>1432.86</v>
+        <v>0</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>-1284.32</v>
+        <v>474.08</v>
       </c>
       <c r="F43" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -5259,7 +5259,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -5269,13 +5269,13 @@
         <v>0</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>474.08</v>
+        <v>0</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0</v>
+        <v>1756.19</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="45">
@@ -5286,23 +5286,23 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>0</v>
+        <v>3155.46</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>0</v>
+        <v>1348.76</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0</v>
+        <v>13692.06</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>1756.19</v>
+        <v>0</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -5313,17 +5313,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>SOPLIN MENDOZA TABITA</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>3155.46</v>
+        <v>0</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>1348.76</v>
+        <v>0</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>13692.06</v>
+        <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
         <v>0</v>
@@ -5340,11 +5340,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>0</v>
+        <v>4237.6</v>
       </c>
       <c r="D47" s="2" t="n">
         <v>0</v>
@@ -5356,7 +5356,7 @@
         <v>0</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="48">
@@ -5367,11 +5367,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>4237.6</v>
+        <v>0</v>
       </c>
       <c r="D48" s="2" t="n">
         <v>0</v>
@@ -5383,7 +5383,7 @@
         <v>0</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="49">
@@ -5394,7 +5394,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -5410,7 +5410,7 @@
         <v>0</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -5421,7 +5421,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -5448,7 +5448,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -5468,46 +5468,19 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>VIVANCO MALDONADO SILVANA MARILY</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G52" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="C53" s="4" t="n">
+      <c r="C52" s="4" t="n">
         <v>35603.86</v>
       </c>
-      <c r="D53" s="4" t="n">
+      <c r="D52" s="4" t="n">
         <v>28143.93</v>
       </c>
-      <c r="E53" s="4" t="n">
+      <c r="E52" s="4" t="n">
         <v>43533.43</v>
       </c>
-      <c r="F53" s="4" t="n">
+      <c r="F52" s="4" t="n">
         <v>2023.29</v>
       </c>
-      <c r="G53" s="4" t="n">
+      <c r="G52" s="4" t="n">
         <v>47200</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-09-09 17:30:21
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2130,10 +2130,10 @@
         <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0</v>
+        <v>436.55</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0</v>
+        <v>417.01</v>
       </c>
       <c r="F28" s="2" t="n">
         <v>0</v>
@@ -2151,13 +2151,13 @@
         <v>0</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>0</v>
+        <v>363.16</v>
       </c>
       <c r="L28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>0</v>
+        <v>1918.73</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
@@ -4043,52 +4043,52 @@
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
+          <t>1 de 58</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>3 de 58</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
           <t>0 de 58</t>
         </is>
       </c>
-      <c r="E60" s="3" t="inlineStr">
-        <is>
-          <t>2 de 58</t>
-        </is>
-      </c>
-      <c r="F60" s="3" t="inlineStr">
+      <c r="G60" s="3" t="inlineStr">
         <is>
           <t>0 de 58</t>
         </is>
       </c>
-      <c r="G60" s="3" t="inlineStr">
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>1 de 58</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>1 de 58</t>
+        </is>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
         <is>
           <t>0 de 58</t>
         </is>
       </c>
-      <c r="H60" s="3" t="inlineStr">
+      <c r="K60" s="3" t="inlineStr">
         <is>
           <t>1 de 58</t>
         </is>
       </c>
-      <c r="I60" s="3" t="inlineStr">
-        <is>
-          <t>1 de 58</t>
-        </is>
-      </c>
-      <c r="J60" s="3" t="inlineStr">
+      <c r="L60" s="3" t="inlineStr">
         <is>
           <t>0 de 58</t>
         </is>
       </c>
-      <c r="K60" s="3" t="inlineStr">
-        <is>
-          <t>0 de 58</t>
-        </is>
-      </c>
-      <c r="L60" s="3" t="inlineStr">
-        <is>
-          <t>0 de 58</t>
-        </is>
-      </c>
       <c r="M60" s="3" t="inlineStr">
         <is>
-          <t>3 de 58</t>
+          <t>4 de 58</t>
         </is>
       </c>
       <c r="N60" s="3" t="inlineStr">
@@ -4819,7 +4819,7 @@
         <v>0</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>598.27</v>
+        <v>5097.28</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>0</v>
@@ -5565,7 +5565,7 @@
         <v>43533.43</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>5231.3</v>
+        <v>9730.309999999999</v>
       </c>
       <c r="G53" s="4" t="n">
         <v>47200</v>
@@ -5589,7 +5589,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5640,13 +5640,13 @@
         <v>2600</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0</v>
+        <v>436.55</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>2600</v>
+        <v>2163.45</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0</v>
+        <v>0.1679038461538462</v>
       </c>
     </row>
     <row r="3">
@@ -5688,13 +5688,13 @@
         <v>199.5</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>271.74</v>
+        <v>688.75</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>-72.24000000000001</v>
+        <v>-489.25</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>1.362105263157895</v>
+        <v>3.452380952380953</v>
       </c>
     </row>
     <row r="5">
@@ -5808,13 +5808,13 @@
         <v>203.76</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0</v>
+        <v>363.16</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>203.76</v>
+        <v>-159.4</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0</v>
+        <v>1.782292893600314</v>
       </c>
     </row>
     <row r="10">
@@ -5832,13 +5832,13 @@
         <v>115</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>39.65</v>
+        <v>1403.21</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>75.34999999999999</v>
+        <v>-1288.21</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.3447826086956521</v>
+        <v>12.20182608695652</v>
       </c>
     </row>
     <row r="11">
@@ -5880,13 +5880,13 @@
         <v>39603</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>4387.43</v>
+        <v>6306.16</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>35215.57</v>
+        <v>33296.84</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.1107852940433806</v>
+        <v>0.1592344014342348</v>
       </c>
     </row>
     <row r="13">
@@ -5899,13 +5899,13 @@
         <v>49040.76</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5297.09</v>
+        <v>9796.1</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>43743.67</v>
+        <v>39244.66</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.1080140275150711</v>
+        <v>0.1997542452441602</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-10 17:30:17
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2085,7 +2085,7 @@
         <v>0</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>0</v>
+        <v>915.36</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0</v>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>3 de 58</t>
+          <t>4 de 58</t>
         </is>
       </c>
       <c r="J60" s="3" t="inlineStr">
@@ -4792,7 +4792,7 @@
         <v>11932.7</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0</v>
+        <v>915.36</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>4000</v>
@@ -5565,7 +5565,7 @@
         <v>43533.43</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>20724.76</v>
+        <v>21640.12</v>
       </c>
       <c r="G53" s="4" t="n">
         <v>47200</v>
@@ -5589,7 +5589,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5760,13 +5760,13 @@
         <v>463</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1196.34</v>
+        <v>2111.7</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-733.3399999999999</v>
+        <v>-1648.7</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>2.583887688984881</v>
+        <v>4.560907127429806</v>
       </c>
     </row>
     <row r="8">
@@ -5899,13 +5899,13 @@
         <v>49040.76</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>20790.55</v>
+        <v>21705.91</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>28250.21</v>
+        <v>27334.85</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.4239442863446651</v>
+        <v>0.4426095761974325</v>
       </c>
     </row>
   </sheetData>

</xml_diff>